<commit_message>
test-40: конвейер 2026-08-28 (run 33153046343)
</commit_message>
<xml_diff>
--- a/output/Тест40_2026-08-28.xlsx
+++ b/output/Тест40_2026-08-28.xlsx
@@ -636,7 +636,11 @@
           <t>Не проверено</t>
         </is>
       </c>
-      <c r="Q2" s="2" t="inlineStr"/>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>совпадает с карточкой</t>
+        </is>
+      </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
           <t>единогласно мед (реестр + 3 судьи)</t>
@@ -720,7 +724,11 @@
           <t>Не проверено</t>
         </is>
       </c>
-      <c r="Q3" s="2" t="inlineStr"/>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>РАСХОЖДЕНИЕ: в карточке 3dformula.ru — на ручную</t>
+        </is>
+      </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
           <t>единогласно мед (реестр + 3 судьи)</t>
@@ -796,7 +804,11 @@
       </c>
       <c r="O4" s="2" t="inlineStr"/>
       <c r="P4" s="2" t="inlineStr"/>
-      <c r="Q4" s="2" t="inlineStr"/>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>РАСХОЖДЕНИЕ: в карточке kzn.3dsystem.ru — на ручную</t>
+        </is>
+      </c>
       <c r="R4" s="2" t="inlineStr">
         <is>
           <t>единогласно мед (реестр + 3 судьи)</t>
@@ -872,7 +884,11 @@
       </c>
       <c r="O5" s="2" t="inlineStr"/>
       <c r="P5" s="2" t="inlineStr"/>
-      <c r="Q5" s="2" t="inlineStr"/>
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>РАСХОЖДЕНИЕ: в карточке rhpnn.ru — на ручную</t>
+        </is>
+      </c>
       <c r="R5" s="2" t="inlineStr">
         <is>
           <t>единогласно мед (реестр + 2 судьи)</t>
@@ -948,7 +964,11 @@
       </c>
       <c r="O6" s="2" t="inlineStr"/>
       <c r="P6" s="2" t="inlineStr"/>
-      <c r="Q6" s="2" t="inlineStr"/>
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>совпадает с карточкой</t>
+        </is>
+      </c>
       <c r="R6" s="2" t="inlineStr">
         <is>
           <t>единогласно мед (реестр + 3 судьи)</t>
@@ -1024,7 +1044,11 @@
       </c>
       <c r="O7" s="2" t="inlineStr"/>
       <c r="P7" s="2" t="inlineStr"/>
-      <c r="Q7" s="2" t="inlineStr"/>
+      <c r="Q7" s="2" t="inlineStr">
+        <is>
+          <t>совпадает с карточкой</t>
+        </is>
+      </c>
       <c r="R7" s="2" t="inlineStr">
         <is>
           <t>единогласно мед (реестр + 3 судьи)</t>
@@ -1063,20 +1087,32 @@
       <c r="G8" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="H8" s="2" t="inlineStr"/>
-      <c r="I8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>a_medika.legal.invitro.ru</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён ИНН</t>
+        </is>
+      </c>
       <c r="J8" s="2" t="inlineStr"/>
       <c r="K8" s="2" t="inlineStr"/>
       <c r="L8" s="2" t="inlineStr"/>
       <c r="M8" s="2" t="inlineStr"/>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Сайт недоступен (уровни 1-4)</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr"/>
       <c r="P8" s="2" t="inlineStr"/>
-      <c r="Q8" s="2" t="inlineStr"/>
+      <c r="Q8" s="2" t="inlineStr">
+        <is>
+          <t>карточка не найдена / без сайта</t>
+        </is>
+      </c>
       <c r="R8" s="2" t="inlineStr">
         <is>
           <t>только реестр: мед-лицензия есть</t>
@@ -1152,7 +1188,11 @@
       </c>
       <c r="O9" s="2" t="inlineStr"/>
       <c r="P9" s="2" t="inlineStr"/>
-      <c r="Q9" s="2" t="inlineStr"/>
+      <c r="Q9" s="2" t="inlineStr">
+        <is>
+          <t>совпадает с карточкой</t>
+        </is>
+      </c>
       <c r="R9" s="2" t="inlineStr">
         <is>
           <t>единогласно мед (реестр + 3 судьи)</t>
@@ -1193,7 +1233,7 @@
       <c r="M10" s="2" t="inlineStr"/>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>сайт не найден</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr"/>
@@ -1274,7 +1314,11 @@
       </c>
       <c r="O11" s="2" t="inlineStr"/>
       <c r="P11" s="2" t="inlineStr"/>
-      <c r="Q11" s="2" t="inlineStr"/>
+      <c r="Q11" s="2" t="inlineStr">
+        <is>
+          <t>совпадает с карточкой</t>
+        </is>
+      </c>
       <c r="R11" s="2" t="inlineStr">
         <is>
           <t>РАСХОЖДЕНИЕ: реестр мед, судьи мед 2/3 — на ручную</t>
@@ -1350,7 +1394,11 @@
       </c>
       <c r="O12" s="2" t="inlineStr"/>
       <c r="P12" s="2" t="inlineStr"/>
-      <c r="Q12" s="2" t="inlineStr"/>
+      <c r="Q12" s="2" t="inlineStr">
+        <is>
+          <t>совпадает с карточкой</t>
+        </is>
+      </c>
       <c r="R12" s="2" t="inlineStr">
         <is>
           <t>единогласно мед (реестр + 3 судьи)</t>
@@ -1426,7 +1474,11 @@
       </c>
       <c r="O13" s="2" t="inlineStr"/>
       <c r="P13" s="2" t="inlineStr"/>
-      <c r="Q13" s="2" t="inlineStr"/>
+      <c r="Q13" s="2" t="inlineStr">
+        <is>
+          <t>РАСХОЖДЕНИЕ: в карточке cheliabinsk.a2med.ru — на ручную</t>
+        </is>
+      </c>
       <c r="R13" s="2" t="inlineStr">
         <is>
           <t>единогласно мед (реестр + 3 судьи)</t>
@@ -1465,23 +1517,51 @@
       <c r="G14" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="H14" s="2" t="inlineStr"/>
-      <c r="I14" s="2" t="inlineStr"/>
-      <c r="J14" s="2" t="inlineStr"/>
-      <c r="K14" s="2" t="inlineStr"/>
-      <c r="L14" s="2" t="inlineStr"/>
-      <c r="M14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>samara.a2med.ru</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён адресом лицензии</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>управляющая компания сети клиник</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>«…d.ru/about/news/deputat-samarskoj-gubernskoj-dumyi-nagradil-sotrudnikov-a2med-za-vklad-v-zdravooxranenie)  [![Image 32: Сеть медицинских центров A2MED успешно провела дебютный выпуск ЦФА](https://samara.a2med.ru/assets/components/phpthumbof/cache/f857ce1a6be64ef2e3a12a7e3650154e.e689433ec902b8707142247a8cb11e8c.jpg) 19.09.2024 #### Сеть медицинских центров A2MED успешно провела деб…» (https://samara.a2med.ru)</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>не похож</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>аллерголог, гастроэнтеролог, гинеколог, дерматолог, иммунолог, кардиолог, косметолог, невролог, онколог, оториноларинголог, офтальмолог, педиатр, ревматолог, стоматолог, терапевт, уролог, флеболог, хирург, эндокринолог</t>
+        </is>
+      </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr"/>
       <c r="P14" s="2" t="inlineStr"/>
-      <c r="Q14" s="2" t="inlineStr"/>
+      <c r="Q14" s="2" t="inlineStr">
+        <is>
+          <t>совпадает с карточкой</t>
+        </is>
+      </c>
       <c r="R14" s="2" t="inlineStr">
         <is>
-          <t>только реестр: мед-лицензия есть</t>
+          <t>единогласно мед (реестр + 3 судьи)</t>
         </is>
       </c>
     </row>
@@ -1554,7 +1634,11 @@
       </c>
       <c r="O15" s="2" t="inlineStr"/>
       <c r="P15" s="2" t="inlineStr"/>
-      <c r="Q15" s="2" t="inlineStr"/>
+      <c r="Q15" s="2" t="inlineStr">
+        <is>
+          <t>карточка не найдена / без сайта</t>
+        </is>
+      </c>
       <c r="R15" s="2" t="inlineStr">
         <is>
           <t>единогласно мед (реестр + 3 судьи)</t>
@@ -1630,7 +1714,11 @@
       </c>
       <c r="O16" s="2" t="inlineStr"/>
       <c r="P16" s="2" t="inlineStr"/>
-      <c r="Q16" s="2" t="inlineStr"/>
+      <c r="Q16" s="2" t="inlineStr">
+        <is>
+          <t>РАСХОЖДЕНИЕ: в карточке donstu.ru — на ручную</t>
+        </is>
+      </c>
       <c r="R16" s="2" t="inlineStr">
         <is>
           <t>единогласно мед (реестр + 3 судьи)</t>
@@ -1706,7 +1794,11 @@
       </c>
       <c r="O17" s="2" t="inlineStr"/>
       <c r="P17" s="2" t="inlineStr"/>
-      <c r="Q17" s="2" t="inlineStr"/>
+      <c r="Q17" s="2" t="inlineStr">
+        <is>
+          <t>совпадает с карточкой</t>
+        </is>
+      </c>
       <c r="R17" s="2" t="inlineStr">
         <is>
           <t>единогласно мед (реестр + 3 судьи)</t>
@@ -1782,7 +1874,11 @@
       </c>
       <c r="O18" s="2" t="inlineStr"/>
       <c r="P18" s="2" t="inlineStr"/>
-      <c r="Q18" s="2" t="inlineStr"/>
+      <c r="Q18" s="2" t="inlineStr">
+        <is>
+          <t>совпадает с карточкой</t>
+        </is>
+      </c>
       <c r="R18" s="2" t="inlineStr">
         <is>
           <t>единогласно мед (реестр + 3 судьи)</t>
@@ -1858,7 +1954,11 @@
       </c>
       <c r="O19" s="2" t="inlineStr"/>
       <c r="P19" s="2" t="inlineStr"/>
-      <c r="Q19" s="2" t="inlineStr"/>
+      <c r="Q19" s="2" t="inlineStr">
+        <is>
+          <t>совпадает с карточкой</t>
+        </is>
+      </c>
       <c r="R19" s="2" t="inlineStr">
         <is>
           <t>единогласно мед (реестр + 3 судьи)</t>
@@ -1934,7 +2034,11 @@
       </c>
       <c r="O20" s="2" t="inlineStr"/>
       <c r="P20" s="2" t="inlineStr"/>
-      <c r="Q20" s="2" t="inlineStr"/>
+      <c r="Q20" s="2" t="inlineStr">
+        <is>
+          <t>карточка не найдена / без сайта</t>
+        </is>
+      </c>
       <c r="R20" s="2" t="inlineStr">
         <is>
           <t>единогласно мед (реестр + 3 судьи)</t>
@@ -2018,7 +2122,11 @@
           <t>Не проверено</t>
         </is>
       </c>
-      <c r="Q21" s="2" t="inlineStr"/>
+      <c r="Q21" s="2" t="inlineStr">
+        <is>
+          <t>совпадает с карточкой</t>
+        </is>
+      </c>
       <c r="R21" s="2" t="inlineStr">
         <is>
           <t>единогласно мед (реестр + 3 судьи)</t>
@@ -2090,7 +2198,11 @@
       </c>
       <c r="O22" s="2" t="inlineStr"/>
       <c r="P22" s="2" t="inlineStr"/>
-      <c r="Q22" s="2" t="inlineStr"/>
+      <c r="Q22" s="2" t="inlineStr">
+        <is>
+          <t>совпадает с карточкой</t>
+        </is>
+      </c>
       <c r="R22" s="2" t="inlineStr">
         <is>
           <t>РАСХОЖДЕНИЕ: реестр мед, судьи мед 0/3 — на ручную</t>
@@ -2137,7 +2249,7 @@
       <c r="M23" s="2" t="inlineStr"/>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>сайт не найден</t>
         </is>
       </c>
       <c r="O23" s="2" t="inlineStr"/>
@@ -2218,7 +2330,11 @@
       </c>
       <c r="O24" s="2" t="inlineStr"/>
       <c r="P24" s="2" t="inlineStr"/>
-      <c r="Q24" s="2" t="inlineStr"/>
+      <c r="Q24" s="2" t="inlineStr">
+        <is>
+          <t>РАСХОЖДЕНИЕ: в карточке aviatraffic.online — на ручную</t>
+        </is>
+      </c>
       <c r="R24" s="2" t="inlineStr">
         <is>
           <t>единогласно мед (реестр + 3 судьи)</t>
@@ -2294,7 +2410,11 @@
       </c>
       <c r="O25" s="2" t="inlineStr"/>
       <c r="P25" s="2" t="inlineStr"/>
-      <c r="Q25" s="2" t="inlineStr"/>
+      <c r="Q25" s="2" t="inlineStr">
+        <is>
+          <t>РАСХОЖДЕНИЕ: в карточке plastic-avismed.ru — на ручную</t>
+        </is>
+      </c>
       <c r="R25" s="2" t="inlineStr">
         <is>
           <t>единогласно мед (реестр + 3 судьи)</t>
@@ -2370,7 +2490,11 @@
       </c>
       <c r="O26" s="2" t="inlineStr"/>
       <c r="P26" s="2" t="inlineStr"/>
-      <c r="Q26" s="2" t="inlineStr"/>
+      <c r="Q26" s="2" t="inlineStr">
+        <is>
+          <t>совпадает с карточкой</t>
+        </is>
+      </c>
       <c r="R26" s="2" t="inlineStr">
         <is>
           <t>единогласно мед (реестр + 3 судьи)</t>
@@ -2446,7 +2570,11 @@
       </c>
       <c r="O27" s="2" t="inlineStr"/>
       <c r="P27" s="2" t="inlineStr"/>
-      <c r="Q27" s="2" t="inlineStr"/>
+      <c r="Q27" s="2" t="inlineStr">
+        <is>
+          <t>РАСХОЖДЕНИЕ: в карточке novosibirsk.mamadeti.ru — на ручную</t>
+        </is>
+      </c>
       <c r="R27" s="2" t="inlineStr">
         <is>
           <t>единогласно мед (реестр + 3 судьи)</t>
@@ -2522,7 +2650,11 @@
       </c>
       <c r="O28" s="2" t="inlineStr"/>
       <c r="P28" s="2" t="inlineStr"/>
-      <c r="Q28" s="2" t="inlineStr"/>
+      <c r="Q28" s="2" t="inlineStr">
+        <is>
+          <t>совпадает с карточкой</t>
+        </is>
+      </c>
       <c r="R28" s="2" t="inlineStr">
         <is>
           <t>единогласно мед (реестр + 3 судьи)</t>
@@ -2598,7 +2730,11 @@
       </c>
       <c r="O29" s="2" t="inlineStr"/>
       <c r="P29" s="2" t="inlineStr"/>
-      <c r="Q29" s="2" t="inlineStr"/>
+      <c r="Q29" s="2" t="inlineStr">
+        <is>
+          <t>карточка не найдена / без сайта</t>
+        </is>
+      </c>
       <c r="R29" s="2" t="inlineStr">
         <is>
           <t>единогласно мед (реестр + 3 судьи)</t>
@@ -2637,23 +2773,47 @@
       <c r="G30" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H30" s="2" t="inlineStr"/>
-      <c r="I30" s="2" t="inlineStr"/>
-      <c r="J30" s="2" t="inlineStr"/>
-      <c r="K30" s="2" t="inlineStr"/>
-      <c r="L30" s="2" t="inlineStr"/>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>rpkavrora.clients.site</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён адресом</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>медицинские слова есть, сильных оснований (лицензия с мед-контекстом / приём врача) нет</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
       <c r="M30" s="2" t="inlineStr"/>
       <c r="N30" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="O30" s="2" t="inlineStr"/>
       <c r="P30" s="2" t="inlineStr"/>
-      <c r="Q30" s="2" t="inlineStr"/>
+      <c r="Q30" s="2" t="inlineStr">
+        <is>
+          <t>совпадает с карточкой</t>
+        </is>
+      </c>
       <c r="R30" s="2" t="inlineStr">
         <is>
-          <t>только реестр: мед-лицензия есть</t>
+          <t>РАСХОЖДЕНИЕ: реестр мед, судьи мед 0/3 — на ручную</t>
         </is>
       </c>
     </row>
@@ -2726,7 +2886,11 @@
       </c>
       <c r="O31" s="2" t="inlineStr"/>
       <c r="P31" s="2" t="inlineStr"/>
-      <c r="Q31" s="2" t="inlineStr"/>
+      <c r="Q31" s="2" t="inlineStr">
+        <is>
+          <t>РАСХОЖДЕНИЕ: в карточке astramed-ms.ru — на ручную</t>
+        </is>
+      </c>
       <c r="R31" s="2" t="inlineStr">
         <is>
           <t>единогласно мед (реестр + 3 судьи)</t>
@@ -2786,7 +2950,11 @@
       </c>
       <c r="O32" s="2" t="inlineStr"/>
       <c r="P32" s="2" t="inlineStr"/>
-      <c r="Q32" s="2" t="inlineStr"/>
+      <c r="Q32" s="2" t="inlineStr">
+        <is>
+          <t>совпадает с карточкой</t>
+        </is>
+      </c>
       <c r="R32" s="2" t="inlineStr">
         <is>
           <t>только реестр: мед-лицензия есть</t>
@@ -2862,7 +3030,11 @@
       </c>
       <c r="O33" s="2" t="inlineStr"/>
       <c r="P33" s="2" t="inlineStr"/>
-      <c r="Q33" s="2" t="inlineStr"/>
+      <c r="Q33" s="2" t="inlineStr">
+        <is>
+          <t>совпадает с карточкой</t>
+        </is>
+      </c>
       <c r="R33" s="2" t="inlineStr">
         <is>
           <t>единогласно мед (реестр + 3 судьи)</t>
@@ -2922,7 +3094,11 @@
       </c>
       <c r="O34" s="2" t="inlineStr"/>
       <c r="P34" s="2" t="inlineStr"/>
-      <c r="Q34" s="2" t="inlineStr"/>
+      <c r="Q34" s="2" t="inlineStr">
+        <is>
+          <t>карточка не найдена / без сайта</t>
+        </is>
+      </c>
       <c r="R34" s="2" t="inlineStr">
         <is>
           <t>только реестр: мед-лицензия есть</t>
@@ -2969,7 +3145,7 @@
       <c r="M35" s="2" t="inlineStr"/>
       <c r="N35" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>сайт не найден</t>
         </is>
       </c>
       <c r="O35" s="2" t="inlineStr"/>
@@ -3050,7 +3226,11 @@
       </c>
       <c r="O36" s="2" t="inlineStr"/>
       <c r="P36" s="2" t="inlineStr"/>
-      <c r="Q36" s="2" t="inlineStr"/>
+      <c r="Q36" s="2" t="inlineStr">
+        <is>
+          <t>РАСХОЖДЕНИЕ: в карточке rostov.agat-group.com — на ручную</t>
+        </is>
+      </c>
       <c r="R36" s="2" t="inlineStr">
         <is>
           <t>единогласно мед (реестр + 3 судьи)</t>
@@ -3097,7 +3277,7 @@
       <c r="M37" s="2" t="inlineStr"/>
       <c r="N37" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>сайт не найден</t>
         </is>
       </c>
       <c r="O37" s="2" t="inlineStr"/>
@@ -3186,7 +3366,11 @@
           <t>Не проверено</t>
         </is>
       </c>
-      <c r="Q38" s="2" t="inlineStr"/>
+      <c r="Q38" s="2" t="inlineStr">
+        <is>
+          <t>совпадает с карточкой</t>
+        </is>
+      </c>
       <c r="R38" s="2" t="inlineStr">
         <is>
           <t>единогласно мед (реестр + 3 судьи)</t>
@@ -3225,23 +3409,51 @@
       <c r="G39" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H39" s="2" t="inlineStr"/>
-      <c r="I39" s="2" t="inlineStr"/>
-      <c r="J39" s="2" t="inlineStr"/>
-      <c r="K39" s="2" t="inlineStr"/>
-      <c r="L39" s="2" t="inlineStr"/>
-      <c r="M39" s="2" t="inlineStr"/>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>smitra.ru</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён адресом лицензии</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>управляющая компания сети клиник</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>«…/news/cherno-belaya-vecherinka-kommersant-sibir-shakhmaty-klassika-i-zabota-o-zdorove-ot-kliniki-smitra/)  [![Image 55: Сеть клиник «Смитра» признана лучшей в здравоохранении на городском конкурсе](https://smitra.ru/upload/webp/upload/iblock/f1d/79x9y5vtvwfiecyksen2q2yv5k2aiqpa.webp)](https://smitra.ru/news/set-klinik-smitra-priznana-luchshey-v-zdravookhranenii-na-goro…» (https://smitra.ru)</t>
+        </is>
+      </c>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>аллерголог, гастроэнтеролог, гинеколог, дерматолог, иммунолог, кардиолог, косметолог, невролог, онколог, отоларинголог, оториноларинголог, офтальмолог, педиатр, психотерапевт, пульмонолог, ревматолог, стоматолог, терапевт, трихолог, уролог, хирург, эндокринолог</t>
+        </is>
+      </c>
       <c r="N39" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="O39" s="2" t="inlineStr"/>
       <c r="P39" s="2" t="inlineStr"/>
-      <c r="Q39" s="2" t="inlineStr"/>
+      <c r="Q39" s="2" t="inlineStr">
+        <is>
+          <t>РАСХОЖДЕНИЕ: в карточке gazpromgr.tomsk.ru — на ручную</t>
+        </is>
+      </c>
       <c r="R39" s="2" t="inlineStr">
         <is>
-          <t>только реестр: мед-лицензия есть</t>
+          <t>единогласно мед (реестр + 3 судьи)</t>
         </is>
       </c>
     </row>
@@ -3314,7 +3526,11 @@
       </c>
       <c r="O40" s="2" t="inlineStr"/>
       <c r="P40" s="2" t="inlineStr"/>
-      <c r="Q40" s="2" t="inlineStr"/>
+      <c r="Q40" s="2" t="inlineStr">
+        <is>
+          <t>совпадает с карточкой</t>
+        </is>
+      </c>
       <c r="R40" s="2" t="inlineStr">
         <is>
           <t>единогласно мед (реестр + 3 судьи)</t>
@@ -3390,7 +3606,11 @@
       </c>
       <c r="O41" s="2" t="inlineStr"/>
       <c r="P41" s="2" t="inlineStr"/>
-      <c r="Q41" s="2" t="inlineStr"/>
+      <c r="Q41" s="2" t="inlineStr">
+        <is>
+          <t>совпадает с карточкой</t>
+        </is>
+      </c>
       <c r="R41" s="2" t="inlineStr">
         <is>
           <t>единогласно мед (реестр + 3 судьи)</t>
@@ -6790,7 +7010,11 @@
           <t>гинекологи, акушерств, кардиологи, неврологи, педиатри, терапи, эндокринологи, гастроэнтерологи, ультразвуковой диагностике, функциональной диагностике, сестринскому делу, эпидемиологи</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>a_medika.legal.invitro.ru</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -6843,7 +7067,11 @@
           <t>онкологи, гинекологи, акушерств, педиатри, терапи, эндокринологи, гастроэнтерологи, ультразвуковой диагностике, функциональной диагностике, сестринскому делу, экспертизе</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>a_medika.legal.invitro.ru</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -6896,7 +7124,11 @@
           <t>гинекологи, акушерств, кардиологи, неврологи, педиатри, терапи, эндокринологи, гастроэнтерологи, ультразвуковой диагностике, функциональной диагностике, сестринскому делу, эпидемиологи</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>a_medika.legal.invitro.ru</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -6941,7 +7173,11 @@
           <t>гинекологи, акушерств, кардиологи, неврологи, оториноларингологи, педиатри, терапи, эндокринологи, гастроэнтерологи, ультразвуковой диагностике, функциональной диагностике, сестринскому делу, эпидемиологи</t>
         </is>
       </c>
-      <c r="K17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>a_medika.legal.invitro.ru</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -6986,7 +7222,11 @@
           <t>косметологи, гинекологи, акушерств, кардиологи, неврологи, педиатри, терапи, эндокринологи, гастроэнтерологи, ультразвуковой диагностике, функциональной диагностике, сестринскому делу, экспертизе</t>
         </is>
       </c>
-      <c r="K18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>a_medika.legal.invitro.ru</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -7039,7 +7279,11 @@
           <t>онкологи, гинекологи, акушерств, кардиологи, неврологи, педиатри, терапи, эндокринологи, гастроэнтерологи, ультразвуковой диагностике, функциональной диагностике, сестринскому делу</t>
         </is>
       </c>
-      <c r="K19" s="2" t="inlineStr"/>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>a_medika.legal.invitro.ru</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -7080,7 +7324,11 @@
           <t>гинекологи, акушерств, кардиологи, неврологи, педиатри, терапи, эндокринологи, гастроэнтерологи, ультразвуковой диагностике, функциональной диагностике, сестринскому делу, экспертизе</t>
         </is>
       </c>
-      <c r="K20" s="2" t="inlineStr"/>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>a_medika.legal.invitro.ru</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -7129,7 +7377,11 @@
           <t>онкологи, гинекологи, акушерств, кардиологи, педиатри, терапи, эндокринологи, гастроэнтерологи, ультразвуковой диагностике, функциональной диагностике, сестринскому делу, экспертизе</t>
         </is>
       </c>
-      <c r="K21" s="2" t="inlineStr"/>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>a_medika.legal.invitro.ru</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -8165,7 +8417,11 @@
           <t>дерматовенерологи, онкологи, гинекологи, акушерств, урологи, кардиологи, неврологи, терапи, хирурги, эндокринологи, гастроэнтерологи, ультразвуковой диагностике, функциональной диагностике, анестезиологии и реаниматологии, сестринскому делу, медицинскому массажу, эпидемиологи, экспертизе</t>
         </is>
       </c>
-      <c r="K41" s="2" t="inlineStr"/>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>samara.a2med.ru</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -8214,7 +8470,11 @@
           <t>онкологи, урологи, кардиологи, неврологи, офтальмологи, оториноларингологи, педиатри, хирурги, травматологии и ортопедии, эндокринологи, гастроэнтерологи, аллергологии и иммунологии, ультразвуковой диагностике, функциональной диагностике, сестринскому делу, медицинскому массажу, эпидемиологи, экспертизе</t>
         </is>
       </c>
-      <c r="K42" s="2" t="inlineStr"/>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>samara.a2med.ru</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -8263,7 +8523,11 @@
           <t>дерматовенерологи, косметологи, онкологи, кардиологи, терапи, эндокринологи, гастроэнтерологи, физиотерапи, ультразвуковой диагностике, сестринскому делу, медицинскому массажу, рефлексотерапи, эпидемиологи, экспертизе</t>
         </is>
       </c>
-      <c r="K43" s="2" t="inlineStr"/>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>samara.a2med.ru</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -8312,7 +8576,11 @@
           <t>анестезиологии и реаниматологии, сестринскому делу</t>
         </is>
       </c>
-      <c r="K44" s="2" t="inlineStr"/>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>samara.a2med.ru</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -8353,7 +8621,11 @@
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr"/>
-      <c r="K45" s="2" t="inlineStr"/>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>samara.a2med.ru</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -14654,7 +14926,11 @@
           <t>косметологи, терапи, физиотерапи, медицинскому массажу, мануальной терапии</t>
         </is>
       </c>
-      <c r="K162" s="2" t="inlineStr"/>
+      <c r="K162" s="2" t="inlineStr">
+        <is>
+          <t>rpkavrora.clients.site</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -15307,7 +15583,11 @@
           <t>дерматовенерологи, онкологи, гинекологи, акушерств, урологи, кардиологи, неврологи, офтальмологи, оториноларингологи, педиатри, терапи, хирурги, травматологии и ортопедии, эндокринологи, гастроэнтерологи, физиотерапи, ультразвуковой диагностике, функциональной диагностике, анестезиологии и реаниматологии, сестринскому делу, медицинскому массажу, эпидемиологи, экспертизе</t>
         </is>
       </c>
-      <c r="K175" s="2" t="inlineStr"/>
+      <c r="K175" s="2" t="inlineStr">
+        <is>
+          <t>smitra.ru</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
@@ -15360,7 +15640,11 @@
           <t>дерматовенерологи, косметологи, онкологи, гинекологи, акушерств, урологи, кардиологи, неврологи, терапи, эндокринологи, гастроэнтерологи, ультразвуковой диагностике, функциональной диагностике, сестринскому делу, эпидемиологи, экспертизе</t>
         </is>
       </c>
-      <c r="K176" s="2" t="inlineStr"/>
+      <c r="K176" s="2" t="inlineStr">
+        <is>
+          <t>smitra.ru</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
@@ -15409,7 +15693,11 @@
           <t>кардиологи, неврологи, офтальмологи, оториноларингологи, педиатри, терапи, травматологии и ортопедии, эндокринологи, гастроэнтерологи, аллергологии и иммунологии, физиотерапи, рентгенологи, ультразвуковой диагностике, сестринскому делу, медицинскому массажу, эпидемиологи, экспертизе</t>
         </is>
       </c>
-      <c r="K177" s="2" t="inlineStr"/>
+      <c r="K177" s="2" t="inlineStr">
+        <is>
+          <t>smitra.ru</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
@@ -15446,7 +15734,11 @@
       <c r="H178" s="2" t="inlineStr"/>
       <c r="I178" s="2" t="inlineStr"/>
       <c r="J178" s="2" t="inlineStr"/>
-      <c r="K178" s="2" t="inlineStr"/>
+      <c r="K178" s="2" t="inlineStr">
+        <is>
+          <t>smitra.ru</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
@@ -15655,7 +15947,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -16489,24 +16781,128 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>А2МЕД, ООО</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>6317157682</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>samara.a2med.ru</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>САЙТ: samara.a2med.ru (страниц скачано: 4)
+TITLE: Медицинский центр А2Мед в Самаре
+МЕНЮ САЙТА (тексты ссылок главной, дословно):
+(ссылок не найдено)
+ЗАГОЛОВКИ h1-h2 (по страницам):
+  (заголовков не найдено)
+КОНТАКТ-БЛОК (строки с ИНН/ОГРН/адресом/лицензией, дословно):
+  https://samara.a2med.ru:
+    «*   [Лицензии](https://samara.a2med.ru/about/licens)»
+    «График работы п. Мехзавод, ул. Николая Баженова, д.6:»
+    «График работы ул. Победы, 69:»
+    «График работы ул. Пугачевский тракт, 80:»
+    «График работы ул. Губанова, 32:»
+    «График работы ул. Лукачева, 10:»
+    «График работы ул. Потапова, 78В:»
+    «График работы ул.Дачная, д.24:»
+    «График работы ул.Партизанская, д.58:»
+    «График работы ул.Мичурина, д.15, 4 этаж:»
+    «График работы ул.Мичурина, д.15, Гинекология, 4 этаж:»
+    «График работы ул.Мичурина, д.15, Детское отделение, 3 этаж:»
+  https://samara.a2med.ru/online-price:
+    «*   [Лицензии](https://samara.a2med.ru/about/licens)»
+    «*    ул. Дачная, д.24»
+    «*    ул. Партизанская, д.58 — **Скидка 10% пенсионерам по средам**»
+    «*    п. Мехзавод, ул. Николая Баженова, д.6»
+    «*    ул. Мичурина, д.15, 4 этаж»
+    «*    ул. Георгия Димитрова, д.90»
+    «*    ул. Революционная, д.125»
+    «*    ул. Пугачевский тракт, д.80»
+    «*    ул. Победы, 69»
+    «*    ул. Победы, 125»
+    «*    ул. Губанова, 32»
+    «*    ул. Лукачева, 10»
+  https://samara.a2med.ru/service:
+    «*   [Лицензии](https://samara.a2med.ru/about/licens)»
+    «График работы п. Мехзавод, ул. Николая Баженова, д.6:»
+    «График работы ул. Победы, 69:»
+    «График работы ул. Пугачевский тракт, 80:»
+    «График работы ул. Губанова, 32:»
+    «График работы ул. Лукачева, 10:»
+    «График работы ул. Потапова, 78В:»
+    «График работы ул.Дачная, д.24:»
+    «График работы ул.Партизанская, д.58:»
+    «График работы ул.Мичурина, д.15, 4 этаж:»
+    «График работы ул.Мичурина, д.15, Гинекология, 4 этаж:»
+    «График работы ул.Мичурина, д.15, Детское отделение, 3 этаж:»
+СПЕЦИАЛЬНОСТИ ВРАЧЕЙ (слова, найденные на страницах): аллерголог, гастроэнтеролог, гинеколог, дерматолог, иммунолог, кардиолог, косметолог, невролог, онколог, оториноларинголог, офтальмолог, педиатр, ревматолог, стоматолог, терапевт, уролог, флеболог, хирург, эндокринолог
+ПРОФИЛЬ-МАРКЕРЫ ДЕРМ-КОНТУРА: дерматолог, дерматология, косметолог, косметология
+ЛИЦЕНЗИЯ (строка с сайта): «Лицензии» (https://samara.a2med.ru)
+ПОЗИЦИИ ПРАЙСА (первые 30 из 82):
+  [Код 02-005] Клинический анализ крови (c лейкоцитарной формулой) (КАК / ОАК / Общий анализ крови) — 230 руб
+  [Код 02-014] Общий анализ крови (без лейкоцитарной формулы и СОЭ) (Гематокрит / Гемоглобин / Лейкоциты / ОАК / Тромбоцит — 160 руб
+  [Код 02-043] Клинический анализ крови: общий анализ, лейкоцитарная формула, СОЭ (с обязательной микроскопией мазка крови — 350 руб
+  [Код 02-006] Общий анализ мочи с микроскопией осадка (КАК / ОАК / Общий анализ крови) — 160 руб
+  [Код 07-025] HBsAg («австралийский» антиген / HBs-антиген / ВГВ / Поверхностный антиген / Вируса гепатита B) — 200 руб
+  [Код 07-009] anti-HCV, антитела (ВГС / Суммарные антитела к вирусу гепатита С) — 410 руб
+  [Код 07-056] Сифилис RPR (антикардиолипиновый тест/микрореакция преципитации), титр (ЛЮЭС / Микрореакция преципитации /  — 140 руб
+  [Код 07-049] Treponema pallidum, антитела (Суммарные антитела к возбудителю сифилиса (бледной трепонеме)) — 290 руб
+  [Код 06-035] Белок общий в сыворотке (Биохимия / Общий белок) — 100 руб
+  [Код 06-036] Билирубин общий (Биохимия / Общий билирубин / Пигмент желчи, продукт распада гемоглобина) — 110 руб
+  [Код 06-034] Мочевина в сыворотке (Конъюгированный билирубин / Связанный билирубин) — 100 руб
+  [Код 40-120] Билирубин и его фракции (общий, прямой и непрямой) (Биохимия) — 120 руб
+  [Код 06-021] Креатинин в сыворотке (с определением СКФ) (1-метилгликоциамидин / Биохимия / Продукт превращения креатинфо — 100 руб
+  [Код 06-033] Мочевая кислота в сыворотке (Биохимия / Продукт метаболизма пуриновых оснований / Пурин-2,6,8-трион) — 110 руб
+  [Код 06-015] Глюкоза в плазме (Биохимия / Сахар крови) — 120 руб
+  [Код 06-014] Гликированный гемоглобин (HbA1c) (Биохимия / Гликозилированный гемоглобин) — 260 руб
+  [Код 06-016] Гомоцистеин (ГЦ / Серосодержащая аминокислота, продукт метаболизма метионина) — 490 руб
+  [Код 06-048] Холестерол общий (Биохимия / Холестерин) — 100 руб
+  [Код 06-028] Холестерол – Липопротеины высокой плотности (ЛПВП) (Альфа-холестерин, липопротеиды высокой плотности / Холе — 130 руб
+  [Код 06-029] Холестерол - Липопротеины низкой плотности (ЛПНП) (Бета-холестерин, липопротеиды низкой плотности / Холесте — 160 руб
+  [Код 06-041] Триглицериды (Липиды крови) — 110 руб
+  [Код 06-012] Витамин В12 (цианокобаламин) (Б12 / Биохимия / Кобаламин / Цианокобаламин) — 350 руб
+  [Код 06-043] Витамин B9 (фолиевая кислота) (Фолаты в сыворотке) — 320 руб
+  [Код 06-106] Витамин D, 25-гидрокси (кальциферол) (25-гидроксивитамин D / 25-гидроксикальциферол / Биохимия / Витамин Д  — 520 руб
+  [Код 06-042] Ферритин (Биохимия / Депонированное железо / Металлопротеид, индикатор запасов железа) — 220 руб
+  [Код 06-040] Трансферрин (Переносчик железа / Сидерофилин) — 230 руб
+  [Код 06-017] Железо в сыворотке (Биохимия / Железо / Ионы железа) — 110 руб
+  [Код 06-018] Железосвязывающая способность сыворотки (Общая железосвязывающая способность сыворотки / ОЖСС) — 170 руб
+  [Код 13-087] Антитела к тиреоглобулину (антиТГ) (АнтиТГ / Проверка функции щитовидной железы / Проверка щитовидной желез — 350 руб
+  [Код 06-020] Кальций в сыворотке (Биохимия / Ионы кальция / Общий кальций) — 110 руб</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>АБВ+, ООО</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>2465176508</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>vesna24.ru</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>САЙТ: vesna24.ru (страниц скачано: 5)
 TITLE: Косметология VESNA в Красноярске, клиника эстетической медицины
@@ -16573,26 +16969,26 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="n">
+    <row r="14">
+      <c r="A14" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>АВ ДГТУ, ООО</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>6165200482</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>аве-вита.рф</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>САЙТ: аве-вита.рф (страниц скачано: 3)
 TITLE: Поликлиника «АвеВита» в Ростове-на-Дону
@@ -16637,26 +17033,26 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="n">
+    <row r="15">
+      <c r="A15" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>АВА-КАЗАНЬ, АО</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>1655146267</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>ava-kazan.ru</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>САЙТ: ava-kazan.ru (страниц скачано: 5)
 TITLE: Клиника внимательной медицины "Скандинавия"
@@ -16747,26 +17143,26 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="n">
+    <row r="16">
+      <c r="A16" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>АВАНТА-МЕД, ООО</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>5406302509</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>avanta-med.ru</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>САЙТ: avanta-med.ru (страниц скачано: 5)
 TITLE: Медицинский центр Аванта-Мед в Новосибирске
@@ -16822,26 +17218,26 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="n">
+    <row r="17">
+      <c r="A17" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>АВАНТИС, ООО</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>5402038349</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>avantis-stom.ru</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>САЙТ: avantis-stom.ru (страниц скачано: 1)
 TITLE: Брекеты в Новосибирске: цена на установку от 14900 рублей
@@ -16869,26 +17265,26 @@
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="n">
+    <row r="18">
+      <c r="A18" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>АВАТАР, ООО</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>7203314735</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>venum-center.ru</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>САЙТ: venum-center.ru (страниц скачано: 1)
 TITLE: Лечение варикоза в Тюмени | Флеболог в Тюмени | УЗИ вен ног в Тюмени | Центр лечения варикоза «Венум»
@@ -16923,26 +17319,26 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="n">
+    <row r="19">
+      <c r="A19" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>АВЕНЮ МЕД, ООО</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>7203527116</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>medlogika.ru</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>САЙТ: medlogika.ru (страниц скачано: 5)
 TITLE: Медицинский центр "МедЛогика" - клиника с добрым сердцем в Тюмени
@@ -17040,26 +17436,26 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="2" t="n">
+    <row r="20">
+      <c r="A20" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>АВЕНЮ, ООО</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>0278947838</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>grandavenue.ru</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>САЙТ: grandavenue.ru (страниц скачано: 1)
 TITLE: Жилой комплекс бизнес-класса для активной жизни в мегаполисе
@@ -17078,26 +17474,26 @@
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="2" t="n">
+    <row r="21">
+      <c r="A21" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>АВИО, ООО ПРЕДПРИЯТИЕ</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>6658006884</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>aviodent.ru</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>САЙТ: aviodent.ru (страниц скачано: 2)
 TITLE: Сеть стоматологических клиник Доктора Мансурского | Платная стоматология в в Екатеринбурге
@@ -17129,26 +17525,26 @@
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="2" t="n">
+    <row r="22">
+      <c r="A22" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>АВИСМЕД, ООО ЛДЦ</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>5406513676</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>avismed-nsk.ru</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>САЙТ: avismed-nsk.ru (страниц скачано: 5)
 TITLE: Лечебно-диагностический центр «АвисМед»
@@ -17195,26 +17591,26 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="2" t="n">
+    <row r="23">
+      <c r="A23" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>АВИЦЕННА-ЭНДОКРИНОЛОГИЯ, ООО</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>1653000230</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>avicenna-endocrin.ru</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>САЙТ: avicenna-endocrin.ru (страниц скачано: 5)
 TITLE: Клиника профессора Анчиковой - Главная
@@ -17274,26 +17670,26 @@
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="2" t="n">
+    <row r="24">
+      <c r="A24" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>АВИЦЕННА, АО МЕДИЦИНСКИЙ ЦЕНТР</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>5406137478</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>avicenna-nsk.ru</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>САЙТ: avicenna-nsk.ru (страниц скачано: 4)
 TITLE: Медицинский центр "АВИЦЕННА" - частная клиника мирового уровня в Новосибирске
@@ -17325,26 +17721,26 @@
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="2" t="n">
+    <row r="25">
+      <c r="A25" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t>АВИЦЕННА, ООО</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="C25" s="2" t="inlineStr">
         <is>
           <t>7204082420</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>avicenna72.ru</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>САЙТ: avicenna72.ru (страниц скачано: 5)
 TITLE: Многопрофильный медицинский центр в Тюмени — «Авиценна»
@@ -17451,26 +17847,26 @@
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="2" t="n">
+    <row r="26">
+      <c r="A26" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>АВК-МЕД, ООО</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>5260156369</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>avk-med.inni.info</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>САЙТ: avk-med.inni.info (страниц скачано: 5)
 TITLE: ООО «АВК-Мед»
@@ -17524,26 +17920,58 @@
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="2" t="n">
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>АВРОРА, ООО</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>6164209193</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>rpkavrora.clients.site</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>САЙТ: rpkavrora.clients.site (страниц скачано: 1)
+TITLE: Типография РПК Аврора
+МЕНЮ САЙТА (тексты ссылок главной, дословно):
+(ссылок не найдено)
+ЗАГОЛОВКИ h1-h2 (по страницам):
+  (заголовков не найдено)
+КОНТАКТ-БЛОК (строки с ИНН/ОГРН/адресом/лицензией, дословно):
+  (не найдено)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
         <v>32</v>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>АВТО-МЕД, ООО</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr">
         <is>
           <t>6324110942</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>флеболог-тольятти.рф</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>САЙТ: флеболог-тольятти.рф (страниц скачано: 1)
 TITLE: Лечение варикоза в Тольятти - приём флеболога, консультация 490 руб.!
@@ -17560,26 +17988,26 @@
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="2" t="n">
+    <row r="29">
+      <c r="A29" s="2" t="n">
         <v>34</v>
       </c>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>АВТОРСКАЯ КЛИНИКА, ООО</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr">
+      <c r="C29" s="2" t="inlineStr">
         <is>
           <t>5407494063</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>avtor-e.ru</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
         <is>
           <t>САЙТ: avtor-e.ru (страниц скачано: 5)
 TITLE: Клиника врачебной косметологии в Новосибирске | Услуги пластической хирургии в авторской клинике доктора Егорова
@@ -17653,26 +18081,26 @@
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="2" t="n">
+    <row r="30">
+      <c r="A30" s="2" t="n">
         <v>37</v>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>АГАТ, ООО</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t>6162081830</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>mc-semya.ru</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>САЙТ: mc-semya.ru (страниц скачано: 5)
 TITLE: Медицинский центр «Семья» в Ростове-на-Дону. Диагностика и лечение.
@@ -17705,26 +18133,26 @@
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="2" t="n">
+    <row r="31">
+      <c r="A31" s="2" t="n">
         <v>39</v>
       </c>
-      <c r="B29" s="2" t="inlineStr">
+      <c r="B31" s="2" t="inlineStr">
         <is>
           <t>АГК, ООО</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>2461016768</t>
         </is>
       </c>
-      <c r="D29" s="2" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>agk24.ru</t>
         </is>
       </c>
-      <c r="E29" s="2" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>САЙТ: agk24.ru (страниц скачано: 5)
 TITLE: Вопросы женского и мужского здоровья | ООО "Андро-гинекологическая клиника", г. Красноярск
@@ -17770,26 +18198,125 @@
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="2" t="n">
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>АДРЕМ, ООО</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>5404465184</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>smitra.ru</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>САЙТ: smitra.ru (страниц скачано: 5)
+TITLE: Многопрофильные клиники «Смитра» в Новосибирске
+МЕНЮ САЙТА (тексты ссылок главной, дословно):
+(ссылок не найдено)
+ЗАГОЛОВКИ h1-h2 (по страницам):
+  (заголовков не найдено)
+КОНТАКТ-БЛОК (строки с ИНН/ОГРН/адресом/лицензией, дословно):
+  https://smitra.ru:
+    «ул. Геодезическая, 2/1, 4, 5, 6 этаж.»
+    «ул. Железнодорожная, 18, 1 и 2 этажи»
+    «ул. Кошурникова, 29/4, 2 этаж.»
+    «Режим работы»
+    «*   [Лицензия](https://smitra.ru/patients/yuridicheskaya-informatsiya/litsenziya-ooo-smk-smitra/ "Лицензия")»
+    «*   [Лицензия](https://smitra.ru/patients/yuridicheskaya-informatsiya/litsenziya-ooo-smk-smitra/)»
+    «ул. Геодезическая, 2/1, 4, 5, 6 этаж.»
+    «ул. Железнодорожная, 18, 1 и 2 этажи»
+    «ул. Кошурникова, 29/4, 2 этаж.»
+    «Режим работы»
+    «ул. Геодезическая, 2/1, 4, 5, 6 этаж.»
+    «ул. Железнодорожная, 18, 1 и 2 этажи»
+  https://smitra.ru/news/novaya-usluga-analiz-na-antitela-igm-k-khantavirusam:
+    «ул. Геодезическая, 2/1, 4, 5, 6 этаж.»
+    «ул. Железнодорожная, 18, 1 и 2 этажи»
+    «ул. Кошурникова, 29/4, 2 этаж.»
+    «Режим работы»
+    «*   [Лицензия](https://smitra.ru/patients/yuridicheskaya-informatsiya/litsenziya-ooo-smk-smitra/ "Лицензия")»
+    «*   [Лицензия](https://smitra.ru/patients/yuridicheskaya-informatsiya/litsenziya-ooo-smk-smitra/)»
+    «ул. Геодезическая, 2/1, 4, 5, 6 этаж.»
+    «ул. Железнодорожная, 18, 1 и 2 этажи»
+    «ул. Кошурникова, 29/4, 2 этаж.»
+    «Режим работы»
+    «ул. Геодезическая, 2/1, 4, 5, 6 этаж.»
+    «ул. Железнодорожная, 18, 1 и 2 этажи»
+  https://smitra.ru/news/novaya-usluga-lechenie-i-omolozhenie-v-ginekologii-lazerom-so-bioxel:
+    «ул. Геодезическая, 2/1, 4, 5, 6 этаж.»
+    «ул. Железнодорожная, 18, 1 и 2 этажи»
+    «ул. Кошурникова, 29/4, 2 этаж.»
+    «Режим работы»
+    «*   [Лицензия](https://smitra.ru/patients/yuridicheskaya-informatsiya/litsenziya-ooo-smk-smitra/ "Лицензия")»
+    «*   [Лицензия](https://smitra.ru/patients/yuridicheskaya-informatsiya/litsenziya-ooo-smk-smitra/)»
+    «ул. Геодезическая, 2/1, 4, 5, 6 этаж.»
+    «ул. Железнодорожная, 18, 1 и 2 этажи»
+    «ул. Кошурникова, 29/4, 2 этаж.»
+    «Режим работы»
+    «ул. Геодезическая, 2/1, 4, 5, 6 этаж.»
+    «ул. Железнодорожная, 18, 1 и 2 этажи»
+  https://smitra.ru/news/novaya-usluga-podbor-kontaktnykh-linz:
+    «ул. Геодезическая, 2/1, 4, 5, 6 этаж.»
+    «ул. Железнодорожная, 18, 1 и 2 этажи»
+    «ул. Кошурникова, 29/4, 2 этаж.»
+    «Режим работы»
+    «*   [Лицензия](https://smitra.ru/patients/yuridicheskaya-informatsiya/litsenziya-ooo-smk-smitra/ "Лицензия")»
+    «*   [Лицензия](https://smitra.ru/patients/yuridicheskaya-informatsiya/litsenziya-ooo-smk-smitra/)»
+    «ул. Геодезическая, 2/1, 4, 5, 6 этаж.»
+    «ул. Железнодорожная, 18, 1 и 2 этажи»
+    «ул. Кошурникова, 29/4, 2 этаж.»
+    «Режим работы»
+    «ул. Геодезическая, 2/1, 4, 5, 6 этаж.»
+    «ул. Железнодорожная, 18, 1 и 2 этажи»
+  https://smitra.ru/patients/bonus/uslugi-s-povyshennym-bonusom:
+    «ул. Геодезическая, 2/1, 4, 5, 6 этаж.»
+    «ул. Железнодорожная, 18, 1 и 2 этажи»
+    «ул. Кошурникова, 29/4, 2 этаж.»
+    «Режим работы»
+    «*   [Лицензия](https://smitra.ru/patients/yuridicheskaya-informatsiya/litsenziya-ooo-smk-smitra/ "Лицензия")»
+    «*   [Лицензия](https://smitra.ru/patients/yuridicheskaya-informatsiya/litsenziya-ooo-smk-smitra/)»
+    «ул. Геодезическая, 2/1, 4, 5, 6 этаж.»
+    «ул. Железнодорожная, 18, 1 и 2 этажи»
+    «ул. Кошурникова, 29/4, 2 этаж.»
+    «Режим работы»
+    «ул. Геодезическая, 2/1, 4, 5, 6 этаж.»
+    «ул. Железнодорожная, 18, 1 и 2 этажи»
+СПЕЦИАЛЬНОСТИ ВРАЧЕЙ (слова, найденные на страницах): аллерголог, гастроэнтеролог, гинеколог, дерматолог, иммунолог, кардиолог, косметолог, невролог, онколог, отоларинголог, оториноларинголог, офтальмолог, педиатр, психотерапевт, пульмонолог, ревматолог, стоматолог, терапевт, трихолог, уролог, хирург, эндокринолог
+ПРОФИЛЬ-МАРКЕРЫ ДЕРМ-КОНТУРА: дерматолог, косметолог, косметология, трихолог
+ЛИЦЕНЗИЯ (строка с сайта): «Лицензия» (https://smitra.ru)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
         <v>41</v>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B33" s="2" t="inlineStr">
         <is>
           <t>АЗБУКА ЗДОРОВЬЯ, ООО</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="C33" s="2" t="inlineStr">
         <is>
           <t>7813610598</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>azbuka-samara.ru</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>САЙТ: azbuka-samara.ru (страниц скачано: 3)
 TITLE: Семейный медицинский центр Самара 🏥 | Детский развивающий клуб
@@ -17822,26 +18349,26 @@
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="2" t="n">
+    <row r="34">
+      <c r="A34" s="2" t="n">
         <v>42</v>
       </c>
-      <c r="B31" s="2" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>АЗБУКА ЗДОРОВЬЯ, ООО</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>6314040975</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>azbuka-samara.ru</t>
         </is>
       </c>
-      <c r="E31" s="2" t="inlineStr">
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>САЙТ: azbuka-samara.ru (страниц скачано: 3)
 TITLE: Семейный медицинский центр Самара 🏥 | Детский развивающий клуб
@@ -17885,7 +18412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H90"/>
+  <dimension ref="A1:H99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -19098,16 +19625,16 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>АБВ+, ООО</t>
+          <t>А2МЕД, ООО</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>2465176508</t>
+          <t>6317157682</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -19122,32 +19649,32 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>не определено</t>
+          <t>управляющая компания сети клиник</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>косметология, онкология, хирургия</t>
+          <t>аллергология, гастроэнтерология, гинекология, дерматология, иммунология, кардиология, косметология, неврология, онкология, оториноларингология, офтальмология, педиатрия, ревматология, стоматология, терапия, урология, флебология, хирургия, эндокринология</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>«Лицензия Л041-01019-24/00338199 от 13.09.2018 г., выдана Министерством здравоохранения Красноярского края»</t>
+          <t>аллерголог, гастроэнтеролог, гинеколог, дерматолог, иммунолог, кардиолог, косметолог, невролог, онколог, оториноларинголог, офтальмолог, педиатр, ревматолог, стоматолог, терапевт, уролог, флеболог, хирург, эндокринолог</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>АБВ+, ООО</t>
+          <t>А2МЕД, ООО</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>2465176508</t>
+          <t>6317157682</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -19162,32 +19689,32 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>не определено</t>
+          <t>управляющая компания сети клиник</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>косметология</t>
+          <t>общая практика, гастроэнтерология, гинекология, дерматология, косметология, стоматология, терапия, хирургия, неврология, кардиология, онкология, офтальмология, педиатрия, ревматология, урология, флебология, иммунология, аллергология, эндокринология, отоларингология</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>Лицензия Л041-01019-24/00338199 от 13.09.2018 г.(действует бессрочно), выдана Министерством здравоохранения Красноярского края</t>
+          <t>График работы ул. Мичурина, д.15, Гинекология, 4 этаж: График работы ул. Мичурина, д.15, Детское отделение, 3 этаж:</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>АБВ+, ООО</t>
+          <t>А2МЕД, ООО</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>2465176508</t>
+          <t>6317157682</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -19202,32 +19729,32 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>не определено</t>
+          <t>управляющая компания сети клиник</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>косметология</t>
+          <t>аллергология, гастроэнтерология, гинекология, дерматология, иммунология, кардиология, косметология, неврология, онкология, оториноларингология, офтальмология, педиатрия, ревматология, стоматология, терапия, урология, флебология, хирургия, эндокринология</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>Лицензированная клиника в Красноярске</t>
+          <t>Медицинский центр А2Мед в Самаре</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>АВ ДГТУ, ООО</t>
+          <t>АБВ+, ООО</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>6165200482</t>
+          <t>2465176508</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -19247,27 +19774,27 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Гинекология, Дерматовенерология, Кардиология, Неврология, Оториноларинология, Офтальмология, Терапия, Урология, Функциональная диагностика, Хирургия, Эндокринология, Стоматология, Гастроэнтерология</t>
+          <t>косметология, онкология, хирургия</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>TITLE: Поликлиника «АвеВита» в Ростове-на-Дону</t>
+          <t>«Лицензия Л041-01019-24/00338199 от 13.09.2018 г., выдана Министерством здравоохранения Красноярского края»</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>АВ ДГТУ, ООО</t>
+          <t>АБВ+, ООО</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>6165200482</t>
+          <t>2465176508</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -19287,27 +19814,27 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>дерматология, венерология</t>
+          <t>косметология</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>Дерматовенеролог, дерматовенерология в профиле врачей и направлениях</t>
+          <t>Лицензия Л041-01019-24/00338199 от 13.09.2018 г.(действует бессрочно), выдана Министерством здравоохранения Красноярского края</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>АВ ДГТУ, ООО</t>
+          <t>АБВ+, ООО</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>6165200482</t>
+          <t>2465176508</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -19327,27 +19854,27 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>гинекология, дерматовенерология, кардиология, неврология, оториноларинология, офтальмология, терапия, урология, функциональная диагностика, хирургия, эндокринология</t>
+          <t>косметология</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>Поликлиника «АвеВита» в Ростове-на-Дону на ул. Текучёва, 145</t>
+          <t>Лицензированная клиника в Красноярске</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>АВА-КАЗАНЬ, АО</t>
+          <t>АВ ДГТУ, ООО</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>1655146267</t>
+          <t>6165200482</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -19362,32 +19889,32 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>медорганизация</t>
+          <t>не определено</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Педиатрия, Диагностика, Гинекология, Оперативная гинекология, Ведение беременности, Гематология, Кардиология, Неврология, Онкология, Маммология, Офтальмология, Флебология, Терапия, Травматология и ортопедия, Урология, Хирургия, Эндокринология, Стационар, Чек‑апы, Детские чек‑апы, Роддом, Реанимация новорожденных, Пластическая хирургия, Косметология, ЭКО, Криоконсервация стволовых клеток из пуповинной крови</t>
+          <t>Гинекология, Дерматовенерология, Кардиология, Неврология, Оториноларинология, Офтальмология, Терапия, Урология, Функциональная диагностика, Хирургия, Эндокринология, Стоматология, Гастроэнтерология</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>Гинекология | Оперативная гинекология | Ведение беременности | Гематология | Кардиология | Неврология | Онкология, маммология</t>
+          <t>TITLE: Поликлиника «АвеВита» в Ростове-на-Дону</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>АВА-КАЗАНЬ, АО</t>
+          <t>АВ ДГТУ, ООО</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>1655146267</t>
+          <t>6165200482</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -19402,32 +19929,32 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>медорганизация</t>
+          <t>не определено</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>гинекология, кардиология, неврология, онкология, офтальмология, флебология, терапия, травматология и ортопедия, урология, хирургия, эндокринология, стоматология, косметология</t>
+          <t>дерматология, венерология</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>Услуги: Гинекология, Кардиология, Неврология, Онкология, Офтальмология, Флебология, Терапия, Травматология и ортопедия, Урология, Хирургия, Эндокринология, Стоматология, Косметология</t>
+          <t>Дерматовенеролог, дерматовенерология в профиле врачей и направлениях</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>АВА-КАЗАНЬ, АО</t>
+          <t>АВ ДГТУ, ООО</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>1655146267</t>
+          <t>6165200482</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -19442,32 +19969,32 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>медорганизация</t>
+          <t>не определено</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>гинекология, педиатрия, диагностика, гематология, кардиология, неврология, онкология, маммология, офтальмология, флебология, терапия, травматология и ортопедия, урология, хирургия, эндокринология, пластическая хирургия, косметология</t>
+          <t>гинекология, дерматовенерология, кардиология, неврология, оториноларинология, офтальмология, терапия, урология, функциональная диагностика, хирургия, эндокринология</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>Клиника внимательной медицины 'Скандинавия'. Записаться на консультацию по номеру 8 (843) 200-10-65 круглосуточно.</t>
+          <t>Поликлиника «АвеВита» в Ростове-на-Дону на ул. Текучёва, 145</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>АВАНТА-МЕД, ООО</t>
+          <t>АВА-КАЗАНЬ, АО</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>5406302509</t>
+          <t>1655146267</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -19487,27 +20014,27 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>гинекология, урология, дерматовенерология, дерматология, подология, отоларингология, сурдология, терапия, гастроэнтерология, хирургия, неврология, эндокринология, сексуология, педиатрия, стоматология, косметология, диагностика</t>
+          <t>Педиатрия, Диагностика, Гинекология, Оперативная гинекология, Ведение беременности, Гематология, Кардиология, Неврология, Онкология, Маммология, Офтальмология, Флебология, Терапия, Травматология и ортопедия, Урология, Хирургия, Эндокринология, Стационар, Чек‑апы, Детские чек‑апы, Роддом, Реанимация новорожденных, Пластическая хирургия, Косметология, ЭКО, Криоконсервация стволовых клеток из пуповинной крови</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>Медицинский центр Аванта-Мед предлагает широкий спектр лечебных и диагностических процедур. Гинекология, урология, отоларингология и другие услуги.</t>
+          <t>Гинекология | Оперативная гинекология | Ведение беременности | Гематология | Кардиология | Неврология | Онкология, маммология</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>АВАНТА-МЕД, ООО</t>
+          <t>АВА-КАЗАНЬ, АО</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>5406302509</t>
+          <t>1655146267</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -19527,27 +20054,27 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>гинекология, урология, дерматология, отоларингология, терапия, гастроэнтерология, хирургия, неврология, эндокринология, сексология, косметология, стоматология</t>
+          <t>гинекология, кардиология, неврология, онкология, офтальмология, флебология, терапия, травматология и ортопедия, урология, хирургия, эндокринология, стоматология, косметология</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>Многопрофильный медицинский центр Аванта-Мед предлагает широкий спектр лечебных и диагностических процедур. Гинекология, урология, отоларингология и другие услуги.</t>
+          <t>Услуги: Гинекология, Кардиология, Неврология, Онкология, Офтальмология, Флебология, Терапия, Травматология и ортопедия, Урология, Хирургия, Эндокринология, Стоматология, Косметология</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>АВАНТА-МЕД, ООО</t>
+          <t>АВА-КАЗАНЬ, АО</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>5406302509</t>
+          <t>1655146267</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -19567,27 +20094,27 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>гинекология, урология, отоларингология, дерматовенерология, дерматология, подология, терапия, гастроэнтерология, хирургия, неврология, эндокринология, сексология, педиатрия, стоматология</t>
+          <t>гинекология, педиатрия, диагностика, гематология, кардиология, неврология, онкология, маммология, офтальмология, флебология, терапия, травматология и ортопедия, урология, хирургия, эндокринология, пластическая хирургия, косметология</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>Многопрофильный медицинский центр Аванта-Мед предлагает широкий спектр лечебных и диагностических процедур. Гинекология, урология, отоларингология и другие услуги.</t>
+          <t>Клиника внимательной медицины 'Скандинавия'. Записаться на консультацию по номеру 8 (843) 200-10-65 круглосуточно.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>АВАНТИС, ООО</t>
+          <t>АВАНТА-МЕД, ООО</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>5402038349</t>
+          <t>5406302509</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -19602,32 +20129,32 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>не определено</t>
+          <t>медорганизация</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>ортодонтия, терапия, хирургия, имплантация, профессиональная чистка, отбеливание, элайнеры</t>
+          <t>гинекология, урология, дерматовенерология, дерматология, подология, отоларингология, сурдология, терапия, гастроэнтерология, хирургия, неврология, эндокринология, сексуология, педиатрия, стоматология, косметология, диагностика</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>Первичная консультация ортодонта — 500 руб</t>
+          <t>Медицинский центр Аванта-Мед предлагает широкий спектр лечебных и диагностических процедур. Гинекология, урология, отоларингология и другие услуги.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>АВАНТИС, ООО</t>
+          <t>АВАНТА-МЕД, ООО</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>5402038349</t>
+          <t>5406302509</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -19642,32 +20169,32 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>не определено</t>
+          <t>медорганизация</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>ортодонтия</t>
+          <t>гинекология, урология, дерматология, отоларингология, терапия, гастроэнтерология, хирургия, неврология, эндокринология, сексология, косметология, стоматология</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>Установка металлических брекетов в Новосибирске по цене 14900 рублей⚡ на одну челюсть. Контрольный приём 7300р. Различные виды металлических, керамических, сапфировых систем.</t>
+          <t>Многопрофильный медицинский центр Аванта-Мед предлагает широкий спектр лечебных и диагностических процедур. Гинекология, урология, отоларингология и другие услуги.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>АВАНТИС, ООО</t>
+          <t>АВАНТА-МЕД, ООО</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>5402038349</t>
+          <t>5406302509</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
@@ -19682,32 +20209,32 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>не определено</t>
+          <t>медорганизация</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>ортодонтия, терапия, хирургия, имплантация</t>
+          <t>гинекология, урология, отоларингология, дерматовенерология, дерматология, подология, терапия, гастроэнтерология, хирургия, неврология, эндокринология, сексология, педиатрия, стоматология</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>Установка металлических брекетов в Новосибирске по цене 14900 рублей⚡ на одну челюсть. Контрольный приём 7300р. Различные виды металлических, керамических, сапфировых систем.</t>
+          <t>Многопрофильный медицинский центр Аванта-Мед предлагает широкий спектр лечебных и диагностических процедур. Гинекология, урология, отоларингология и другие услуги.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>АВАТАР, ООО</t>
+          <t>АВАНТИС, ООО</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>7203314735</t>
+          <t>5402038349</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -19722,32 +20249,32 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>медорганизация</t>
+          <t>не определено</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>флебология, хирургия</t>
+          <t>ортодонтия, терапия, хирургия, имплантация, профессиональная чистка, отбеливание, элайнеры</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>«Лицензия № Л041-01107-72/00361525»</t>
+          <t>Первичная консультация ортодонта — 500 руб</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>АВАТАР, ООО</t>
+          <t>АВАНТИС, ООО</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>7203314735</t>
+          <t>5402038349</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -19762,32 +20289,32 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>медорганизация</t>
+          <t>не определено</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>флебология</t>
+          <t>ортодонтия</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>Лицензия № Л041-01107-72/00361525 на медицинскую деятельность, приём врача-флеболога, медицинские услуги в прайсе</t>
+          <t>Установка металлических брекетов в Новосибирске по цене 14900 рублей⚡ на одну челюсть. Контрольный приём 7300р. Различные виды металлических, керамических, сапфировых систем.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>АВАТАР, ООО</t>
+          <t>АВАНТИС, ООО</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>7203314735</t>
+          <t>5402038349</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -19802,32 +20329,32 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>медорганизация</t>
+          <t>не определено</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>флебология, хирургия</t>
+          <t>ортодонтия, терапия, хирургия, имплантация</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>Лицензия № Л041-01107-72/00361525, приём врача-флеболога, лазерное лечение варикоза, склеротерапия, перевязка при трофической язве</t>
+          <t>Установка металлических брекетов в Новосибирске по цене 14900 рублей⚡ на одну челюсть. Контрольный приём 7300р. Различные виды металлических, керамических, сапфировых систем.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>АВЕНЮ МЕД, ООО</t>
+          <t>АВАТАР, ООО</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>7203527116</t>
+          <t>7203314735</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -19842,32 +20369,32 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>не определено</t>
+          <t>медорганизация</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>гастроэнтерология, гинекология, кардиология, неврология, педиатрия, ревматология, терапия, урология, хирургия, эндокринология, ультразвуковая диагностика, функциональная диагностика, нутрициология, психология</t>
+          <t>флебология, хирургия</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>Гинеколог, врач УЗИ, детский гинеколог — 2 000 ₽</t>
+          <t>«Лицензия № Л041-01107-72/00361525»</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>АВЕНЮ МЕД, ООО</t>
+          <t>АВАТАР, ООО</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>7203527116</t>
+          <t>7203314735</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -19882,32 +20409,32 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>не определено</t>
+          <t>медорганизация</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>акушерство и гинекология, кардиология, неврология, терапия, гастроэнтерология, урология, хирургия, эндокринология, психология, nutriциология</t>
+          <t>флебология</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>2021 г. — "Акушерство и гинекология", Тюменский государственный медицинский университет</t>
+          <t>Лицензия № Л041-01107-72/00361525 на медицинскую деятельность, приём врача-флеболога, медицинские услуги в прайсе</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>АВЕНЮ МЕД, ООО</t>
+          <t>АВАТАР, ООО</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>7203527116</t>
+          <t>7203314735</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -19922,32 +20449,32 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>не определено</t>
+          <t>медорганизация</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>гастроэнтерология, гинекология, кардиология, неврология, педиатрия, ревматология, терапия, урология, хирургия, эндокринология</t>
+          <t>флебология, хирургия</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>Медицинский центр 'МедЛогика' - клиника с добрым сердцем в Тюмени. Лицензии и сертификаты доступны на сайте. Указаны медицинские специалисты и услуги.</t>
+          <t>Лицензия № Л041-01107-72/00361525, приём врача-флеболога, лазерное лечение варикоза, склеротерапия, перевязка при трофической язве</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>АВЕНЮ, ООО</t>
+          <t>АВЕНЮ МЕД, ООО</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>0278947838</t>
+          <t>7203527116</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -19957,33 +20484,37 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>не медорганизация</t>
+          <t>медорганизация</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>не медорганизация</t>
-        </is>
-      </c>
-      <c r="G52" s="2" t="inlineStr"/>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>гастроэнтерология, гинекология, кардиология, неврология, педиатрия, ревматология, терапия, урология, хирургия, эндокринология, ультразвуковая диагностика, функциональная диагностика, нутрициология, психология</t>
+        </is>
+      </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>Жилой комплекс бизнес-класса для активной жизни в мегаполисе</t>
+          <t>Гинеколог, врач УЗИ, детский гинеколог — 2 000 ₽</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>АВЕНЮ, ООО</t>
+          <t>АВЕНЮ МЕД, ООО</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>0278947838</t>
+          <t>7203527116</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
@@ -19993,33 +20524,37 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>не медорганизация</t>
+          <t>медорганизация</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>не медорганизация</t>
-        </is>
-      </c>
-      <c r="G53" s="2" t="inlineStr"/>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>акушерство и гинекология, кардиология, неврология, терапия, гастроэнтерология, урология, хирургия, эндокринология, психология, nutriциология</t>
+        </is>
+      </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>TITLE: Жилой комплекс бизнес-класса для активной жизни в мегаполисе</t>
+          <t>2021 г. — "Акушерство и гинекология", Тюменский государственный медицинский университет</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>АВЕНЮ, ООО</t>
+          <t>АВЕНЮ МЕД, ООО</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>0278947838</t>
+          <t>7203527116</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
@@ -20029,33 +20564,37 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>не медорганизация</t>
+          <t>медорганизация</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>не медорганизация</t>
-        </is>
-      </c>
-      <c r="G54" s="2" t="inlineStr"/>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>гастроэнтерология, гинекология, кардиология, неврология, педиатрия, ревматология, терапия, урология, хирургия, эндокринология</t>
+        </is>
+      </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>Жилой комплекс бизнес-класса для активной жизни в мегаполисе</t>
+          <t>Медицинский центр 'МедЛогика' - клиника с добрым сердцем в Тюмени. Лицензии и сертификаты доступны на сайте. Указаны медицинские специалисты и услуги.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>АВИО, ООО ПРЕДПРИЯТИЕ</t>
+          <t>АВЕНЮ, ООО</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>6658006884</t>
+          <t>0278947838</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
@@ -20065,37 +20604,33 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>медорганизация</t>
+          <t>не медорганизация</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>не определено</t>
-        </is>
-      </c>
-      <c r="G55" s="2" t="inlineStr">
-        <is>
-          <t>стоматология, детская стоматология, имплантация, протезирование, пародонтология, гигиена, хирургия, ортопедическая стоматология</t>
-        </is>
-      </c>
+          <t>не медорганизация</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr"/>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>Сеть стоматологических клиник Доктора Мансурского - все виды стоматологических услуг в Москве. Цены на прием в стоматологии, запись на прием он-лайн.</t>
+          <t>Жилой комплекс бизнес-класса для активной жизни в мегаполисе</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>АВИО, ООО ПРЕДПРИЯТИЕ</t>
+          <t>АВЕНЮ, ООО</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>6658006884</t>
+          <t>0278947838</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
@@ -20105,37 +20640,33 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>медорганизация</t>
+          <t>не медорганизация</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>не определено</t>
-        </is>
-      </c>
-      <c r="G56" s="2" t="inlineStr">
-        <is>
-          <t>стоматология</t>
-        </is>
-      </c>
+          <t>не медорганизация</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr"/>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>Сеть стоматологических клиник Доктора Мансурского - все виды стоматологических услуг в Москве. Цены на прием в стоматологии, запись на прием он-лайн. Платная зубная клиника</t>
+          <t>TITLE: Жилой комплекс бизнес-класса для активной жизни в мегаполисе</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>АВИО, ООО ПРЕДПРИЯТИЕ</t>
+          <t>АВЕНЮ, ООО</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>6658006884</t>
+          <t>0278947838</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
@@ -20145,37 +20676,33 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>медорганизация</t>
+          <t>не медорганизация</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>не определено</t>
-        </is>
-      </c>
-      <c r="G57" s="2" t="inlineStr">
-        <is>
-          <t>стоматология</t>
-        </is>
-      </c>
+          <t>не медорганизация</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr"/>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>Сеть стоматологических клиник Доктора Мансурского - все виды стоматологических услуг в Москве. Цены на прием в стоматологии, запись на прием он-лайн. Платная зубная клиника</t>
+          <t>Жилой комплекс бизнес-класса для активной жизни в мегаполисе</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>АВИСМЕД, ООО ЛДЦ</t>
+          <t>АВИО, ООО ПРЕДПРИЯТИЕ</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>5406513676</t>
+          <t>6658006884</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
@@ -20190,32 +20717,32 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>медорганизация</t>
+          <t>не определено</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Диагностическое отделение, Консультативное отделение, Косметологическое отделение, Педиатрическое отделение, Хирургическое отделение</t>
+          <t>стоматология, детская стоматология, имплантация, протезирование, пародонтология, гигиена, хирургия, ортопедическая стоматология</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>Лечебно-диагностический центр «АвисМед»</t>
+          <t>Сеть стоматологических клиник Доктора Мансурского - все виды стоматологических услуг в Москве. Цены на прием в стоматологии, запись на прием он-лайн.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>АВИСМЕД, ООО ЛДЦ</t>
+          <t>АВИО, ООО ПРЕДПРИЯТИЕ</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>5406513676</t>
+          <t>6658006884</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -20230,32 +20757,32 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>медорганизация</t>
+          <t>не определено</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>дерматология, косметология</t>
+          <t>стоматология</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>Лечебно-диагностический центр «АвисМед», специалисты: гинеколог, дерматолог, косметолог, невролог, онколог, оториноларинголог, педиатр, стоматолог, терапевт, уролог, флеболог, хирург</t>
+          <t>Сеть стоматологических клиник Доктора Мансурского - все виды стоматологических услуг в Москве. Цены на прием в стоматологии, запись на прием он-лайн. Платная зубная клиника</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>АВИСМЕД, ООО ЛДЦ</t>
+          <t>АВИО, ООО ПРЕДПРИЯТИЕ</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>5406513676</t>
+          <t>6658006884</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
@@ -20270,32 +20797,32 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>медорганизация</t>
+          <t>не определено</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>гинекология, дерматология, косметология, неврология, онкология, оториноларингология, педиатрия, стоматология, терапия, урология, флебология, хирургия</t>
+          <t>стоматология</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>Записаться на услуги лечебно-диагностического центра «АвисМед»</t>
+          <t>Сеть стоматологических клиник Доктора Мансурского - все виды стоматологических услуг в Москве. Цены на прием в стоматологии, запись на прием он-лайн. Платная зубная клиника</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>АВИЦЕННА-ЭНДОКРИНОЛОГИЯ, ООО</t>
+          <t>АВИСМЕД, ООО ЛДЦ</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>1653000230</t>
+          <t>5406513676</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
@@ -20310,32 +20837,32 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>не определено</t>
+          <t>медорганизация</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>эндокринология, детская эндокринология, кардиология, терапия, ультразвуковая диагностика, гастроэнтерология, детская гастроэнтерология, андрология‑урология, детская урология‑андрология, акушер‑гинекология, детская акушер‑гинекология, неврология, детская неврология, остеопатия, детская остеопатия, мануальная терапия, сосудистый хирург‑флебология, онкология, маммология, хирургия (включая ожоговый хирург), нефрология, детская нефрология, психотерапия, детская психотерапия, массаж, нутрициология, офтальмология, детская офтальмология, функциональная диагностика, травматология‑ортопедия, педиатрия, дерматология, детская дерматология, генетические исследования, криодеструкция, биоимпедансометрия, физиотерапия, озонотерапия, склеротерапия, краниосакральная терапия</t>
+          <t>Диагностическое отделение, Консультативное отделение, Косметологическое отделение, Педиатрическое отделение, Хирургическое отделение</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>Клиника профессора Анчиковой. Опыт работы более 25 лет</t>
+          <t>Лечебно-диагностический центр «АвисМед»</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>АВИЦЕННА-ЭНДОКРИНОЛОГИЯ, ООО</t>
+          <t>АВИСМЕД, ООО ЛДЦ</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>1653000230</t>
+          <t>5406513676</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -20350,32 +20877,32 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>не определено</t>
+          <t>медорганизация</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>эндокринология, гастроэнтерология, гинекология, дерматология, кардиология, неврология, онкология, офтальмология, педиатрия, психотерапия, терапия, урология, флебология, хирургия</t>
+          <t>дерматология, косметология</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>Услуги: Эндокринолог, Гастроэнтеролог, Гинеколог, Дерматолог, Кардиолог, Невролог, Онколог, Офтальмолог, Педиатр, Психотерапевт, Терапевт, Уролог, Флеболог, Хирург</t>
+          <t>Лечебно-диагностический центр «АвисМед», специалисты: гинеколог, дерматолог, косметолог, невролог, онколог, оториноларинголог, педиатр, стоматолог, терапевт, уролог, флеболог, хирург</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>АВИЦЕННА-ЭНДОКРИНОЛОГИЯ, ООО</t>
+          <t>АВИСМЕД, ООО ЛДЦ</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>1653000230</t>
+          <t>5406513676</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
@@ -20390,32 +20917,32 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>не определено</t>
+          <t>медорганизация</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>эндокринология, гастроэнтерология, гинекология, дерматология, кардиология, неврология, онкология, офтальмология, педиатрия, психотерапия, терапия, урология, флебология, хирургия</t>
+          <t>гинекология, дерматология, косметология, неврология, онкология, оториноларингология, педиатрия, стоматология, терапия, урология, флебология, хирургия</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>Клиника профессора Анчиковой. Опыт работы более 25 лет</t>
+          <t>Записаться на услуги лечебно-диагностического центра «АвисМед»</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>АВИЦЕННА, АО МЕДИЦИНСКИЙ ЦЕНТР</t>
+          <t>АВИЦЕННА-ЭНДОКРИНОЛОГИЯ, ООО</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>5406137478</t>
+          <t>1653000230</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
@@ -20435,27 +20962,27 @@
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>гинекология, кардиология и сердечно‑сосудистая хирургия, неврология и нейрохирургия, травматология и ортопедия, урология, онкология, оториноларингология, офтальмология и микрохирургия глаза, пластическая и реконструктивная хирургия, педиатрия, терапия, стоматология, лечения бесплодия (ЭКО), лабораторная и генетическая диагностика, лучевая диагностика, восстановительное лечение</t>
+          <t>эндокринология, детская эндокринология, кардиология, терапия, ультразвуковая диагностика, гастроэнтерология, детская гастроэнтерология, андрология‑урология, детская урология‑андрология, акушер‑гинекология, детская акушер‑гинекология, неврология, детская неврология, остеопатия, детская остеопатия, мануальная терапия, сосудистый хирург‑флебология, онкология, маммология, хирургия (включая ожоговый хирург), нефрология, детская нефрология, психотерапия, детская психотерапия, массаж, нутрициология, офтальмология, детская офтальмология, функциональная диагностика, травматология‑ортопедия, педиатрия, дерматология, детская дерматология, генетические исследования, криодеструкция, биоимпедансометрия, физиотерапия, озонотерапия, склеротерапия, краниосакральная терапия</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>TITLE: Медицинский центр "АВИЦЕННА" - частная клиника мирового уровня в Новосибирске; меню сайта содержит разделы «Клиника гинекологическое», «Клиника кардиологии», «Клиника неврологии», «Клиника онкологии» и др., а также ссылки «Лицензии».</t>
+          <t>Клиника профессора Анчиковой. Опыт работы более 25 лет</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>АВИЦЕННА, АО МЕДИЦИНСКИЙ ЦЕНТР</t>
+          <t>АВИЦЕННА-ЭНДОКРИНОЛОГИЯ, ООО</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>5406137478</t>
+          <t>1653000230</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
@@ -20475,27 +21002,27 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>гинекология, неврология и нейрохирургия, офтальмология и микрохирургия глаза, общая хирургия, пластическая хирургия, ведение беременности и роды, травматология и ортопедия, лабораторная и генетическая диагностика, педиатрия, терапия, урология, онкология, кардиология и сердечно-сосудистая хирургия, оториноларингология</t>
+          <t>эндокринология, гастроэнтерология, гинекология, дерматология, кардиология, неврология, онкология, офтальмология, педиатрия, психотерапия, терапия, урология, флебология, хирургия</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>Направления деятельности</t>
+          <t>Услуги: Эндокринолог, Гастроэнтеролог, Гинеколог, Дерматолог, Кардиолог, Невролог, Онколог, Офтальмолог, Педиатр, Психотерапевт, Терапевт, Уролог, Флеболог, Хирург</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>АВИЦЕННА, АО МЕДИЦИНСКИЙ ЦЕНТР</t>
+          <t>АВИЦЕННА-ЭНДОКРИНОЛОГИЯ, ООО</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>5406137478</t>
+          <t>1653000230</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
@@ -20515,27 +21042,27 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>гинекология, неврология и нейрохирургия, офтальмология и микрохирургия глаза, лечение бесплодия (ЭКО), общая хирургия, пластическая хирургия, ведение беременности и роды, травматология и ортопедия, лабораторная и генетическая диагностика, педиатрия, лучевая диагностика, терапия, урология, ультразвуковая диагностика, стоматология, онкология, восстановительное лечение, кардиология и сердечно-сосудистая хирургия, оториноларингология</t>
+          <t>эндокринология, гастроэнтерология, гинекология, дерматология, кардиология, неврология, онкология, офтальмология, педиатрия, психотерапия, терапия, урология, флебология, хирургия</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>Медицинский центр 'АВИЦЕННА' - частная клиника мирового уровня в Новосибирске</t>
+          <t>Клиника профессора Анчиковой. Опыт работы более 25 лет</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>АВИЦЕННА, ООО</t>
+          <t>АВИЦЕННА, АО МЕДИЦИНСКИЙ ЦЕНТР</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>7204082420</t>
+          <t>5406137478</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
@@ -20550,32 +21077,32 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>медорганизация</t>
+          <t>не определено</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>Аллергология и иммунология, Акушерство и гинекология, Гастроэнтерология, Дерматовенерология / дерматология, Кардиология, Неврология, Отоларингология (ЛОР), Офтальмология, Подология, Пульмонология, Ревматология, Рентгенологические исследования, Стоматология, Терапия (общая), Трихология, УЗИ диагностика, Урология, Физиотерапия, Фитотерапия, Эндокринология, Гирудотерапия, Криотерапия, Лабораторная диагностика, Функциональная диагностика</t>
+          <t>гинекология, кардиология и сердечно‑сосудистая хирургия, неврология и нейрохирургия, травматология и ортопедия, урология, онкология, оториноларингология, офтальмология и микрохирургия глаза, пластическая и реконструктивная хирургия, педиатрия, терапия, стоматология, лечения бесплодия (ЭКО), лабораторная и генетическая диагностика, лучевая диагностика, восстановительное лечение</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>Лицензия № Л041-01107-72/00367188 от 16.11.2018 г. на осуществление Медицинской деятельности.</t>
+          <t>TITLE: Медицинский центр "АВИЦЕННА" - частная клиника мирового уровня в Новосибирске; меню сайта содержит разделы «Клиника гинекологическое», «Клиника кардиологии», «Клиника неврологии», «Клиника онкологии» и др., а также ссылки «Лицензии».</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>АВИЦЕННА, ООО</t>
+          <t>АВИЦЕННА, АО МЕДИЦИНСКИЙ ЦЕНТР</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>7204082420</t>
+          <t>5406137478</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
@@ -20590,32 +21117,32 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>медорганизация</t>
+          <t>не определено</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>аллергология, гинекология</t>
+          <t>гинекология, неврология и нейрохирургия, офтальмология и микрохирургия глаза, общая хирургия, пластическая хирургия, ведение беременности и роды, травматология и ортопедия, лабораторная и генетическая диагностика, педиатрия, терапия, урология, онкология, кардиология и сердечно-сосудистая хирургия, оториноларингология</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>Лицензия № Л041-01107-72/00367188 от 16.11.2018 г. на осуществление Медицинской деятельности</t>
+          <t>Направления деятельности</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>АВИЦЕННА, ООО</t>
+          <t>АВИЦЕННА, АО МЕДИЦИНСКИЙ ЦЕНТР</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>7204082420</t>
+          <t>5406137478</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
@@ -20630,32 +21157,32 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>медорганизация</t>
+          <t>не определено</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>аллергология-иммунология, акушерство-гинекология, гастроэнтерология, дерматовенерология, кардиология, неврология, отоларингология, офтальмология, пульмонология, ревматология, стоматология, терапия, эндокринология</t>
+          <t>гинекология, неврология и нейрохирургия, офтальмология и микрохирургия глаза, лечение бесплодия (ЭКО), общая хирургия, пластическая хирургия, ведение беременности и роды, травматология и ортопедия, лабораторная и генетическая диагностика, педиатрия, лучевая диагностика, терапия, урология, ультразвуковая диагностика, стоматология, онкология, восстановительное лечение, кардиология и сердечно-сосудистая хирургия, оториноларингология</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>Лицензия № Л041-01107-72/00367188 от 16.11.2018 г. на осуществление Медицинской деятельности.</t>
+          <t>Медицинский центр 'АВИЦЕННА' - частная клиника мирового уровня в Новосибирске</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>АВК-МЕД, ООО</t>
+          <t>АВИЦЕННА, ООО</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>5260156369</t>
+          <t>7204082420</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
@@ -20670,32 +21197,32 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>не определено</t>
+          <t>медорганизация</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>иммунология, терапия, хирургия, кардиология, гастроэнтерология, лабораторная диагностика</t>
+          <t>Аллергология и иммунология, Акушерство и гинекология, Гастроэнтерология, Дерматовенерология / дерматология, Кардиология, Неврология, Отоларингология (ЛОР), Офтальмология, Подология, Пульмонология, Ревматология, Рентгенологические исследования, Стоматология, Терапия (общая), Трихология, УЗИ диагностика, Урология, Физиотерапия, Фитотерапия, Эндокринология, Гирудотерапия, Криотерапия, Лабораторная диагностика, Функциональная диагностика</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>Специальности врачей: иммунолог, терапевт, хирург; позиции прайса включают Болезнь Крона, Артериальная гипертония, анализы крови и другие медицинские услуги.</t>
+          <t>Лицензия № Л041-01107-72/00367188 от 16.11.2018 г. на осуществление Медицинской деятельности.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>АВК-МЕД, ООО</t>
+          <t>АВИЦЕННА, ООО</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>5260156369</t>
+          <t>7204082420</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
@@ -20710,32 +21237,32 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>не определено</t>
+          <t>медорганизация</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>иммунология, терапия, хирургия, кардиология</t>
+          <t>аллергология, гинекология</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>Позиции прайса: Болезнь Крона, Артериальная гипертония, Атеросклероз, Профиль №45 "Сердечно-сосудистые заболевания"</t>
+          <t>Лицензия № Л041-01107-72/00367188 от 16.11.2018 г. на осуществление Медицинской деятельности</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>АВК-МЕД, ООО</t>
+          <t>АВИЦЕННА, ООО</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>5260156369</t>
+          <t>7204082420</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
@@ -20750,32 +21277,32 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>не определено</t>
+          <t>медорганизация</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>иммунология, терапия, хирургия</t>
+          <t>аллергология-иммунология, акушерство-гинекология, гастроэнтерология, дерматовенерология, кардиология, неврология, отоларингология, офтальмология, пульмонология, ревматология, стоматология, терапия, эндокринология</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>https://avk-med.inni.info/produkt/meditsinskiye-uslugi-analizy-meditsinskiye: «ул. Ошарская, д.14-В»</t>
+          <t>Лицензия № Л041-01107-72/00367188 от 16.11.2018 г. на осуществление Медицинской деятельности.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>АВТО-МЕД, ООО</t>
+          <t>АВК-МЕД, ООО</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>6324110942</t>
+          <t>5260156369</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
@@ -20790,32 +21317,32 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>медорганизация</t>
+          <t>не определено</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>флебология, хирургия</t>
+          <t>иммунология, терапия, хирургия, кардиология, гастроэнтерология, лабораторная диагностика</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>Лечение варикоза в Тольятти - приём флеболога, консультация 490 руб.</t>
+          <t>Специальности врачей: иммунолог, терапевт, хирург; позиции прайса включают Болезнь Крона, Артериальная гипертония, анализы крови и другие медицинские услуги.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>АВТО-МЕД, ООО</t>
+          <t>АВК-МЕД, ООО</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>6324110942</t>
+          <t>5260156369</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
@@ -20830,32 +21357,32 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>медорганизация</t>
+          <t>не определено</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>флебология</t>
+          <t>иммунология, терапия, хирургия, кардиология</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>Лечение варикоза в Тольятти - приём флеболога, консультация 490 руб.</t>
+          <t>Позиции прайса: Болезнь Крона, Артериальная гипертония, Атеросклероз, Профиль №45 "Сердечно-сосудистые заболевания"</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>АВТО-МЕД, ООО</t>
+          <t>АВК-МЕД, ООО</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>6324110942</t>
+          <t>5260156369</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
@@ -20870,32 +21397,32 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>медорганизация</t>
+          <t>не определено</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>флебология, хирургия</t>
+          <t>иммунология, терапия, хирургия</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>Лечение варикоза в Тольятти - приём флеболога, консультация 490 руб!</t>
+          <t>https://avk-med.inni.info/produkt/meditsinskiye-uslugi-analizy-meditsinskiye: «ул. Ошарская, д.14-В»</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>АВТОРСКАЯ КЛИНИКА, ООО</t>
+          <t>АВРОРА, ООО</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>5407494063</t>
+          <t>6164209193</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
@@ -20905,7 +21432,7 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>медорганизация</t>
+          <t>не определено</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
@@ -20913,29 +21440,25 @@
           <t>не определено</t>
         </is>
       </c>
-      <c r="G76" s="2" t="inlineStr">
-        <is>
-          <t>пластическая хирургия, косметология, диетология, сомнология, мезотерапия, пилинг, инъекционная косметология, аппаратная косметология, хирургия груди, хирургия тела, хирургия лица, биоимпедансометрия, похудение</t>
-        </is>
-      </c>
+      <c r="G76" s="2" t="inlineStr"/>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>Клиника пластической хирургии и врачебной косметологии в Новосибирске</t>
+          <t>TITLE: Типография РПК Аврора</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>АВТОРСКАЯ КЛИНИКА, ООО</t>
+          <t>АВРОРА, ООО</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>5407494063</t>
+          <t>6164209193</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
@@ -20945,7 +21468,7 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>медорганизация</t>
+          <t>не медорганизация</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
@@ -20953,29 +21476,25 @@
           <t>не определено</t>
         </is>
       </c>
-      <c r="G77" s="2" t="inlineStr">
-        <is>
-          <t>косметология, пластическая хирургия</t>
-        </is>
-      </c>
+      <c r="G77" s="2" t="inlineStr"/>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>Лицензия №1, Приложение к лицензии №1, Приложение к лицензии №2-1, Приложение к лицензии №2-2, Приложение к лицензии №2-3, Лицензия №2</t>
+          <t>TITLE: Типография РПК Аврора</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>АВТОРСКАЯ КЛИНИКА, ООО</t>
+          <t>АВРОРА, ООО</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>5407494063</t>
+          <t>6164209193</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
@@ -20985,7 +21504,7 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>медорганизация</t>
+          <t>не медорганизация</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
@@ -20993,29 +21512,25 @@
           <t>не определено</t>
         </is>
       </c>
-      <c r="G78" s="2" t="inlineStr">
-        <is>
-          <t>пластическая хирургия, врачебная косметология, диетология, сомнология</t>
-        </is>
-      </c>
+      <c r="G78" s="2" t="inlineStr"/>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>Клиника пластической хирургии и врачебной косметологии в Новосибирске</t>
+          <t>Типография РПК Аврора</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>АГАТ, ООО</t>
+          <t>АВТО-МЕД, ООО</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>6162081830</t>
+          <t>6324110942</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
@@ -21030,32 +21545,32 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>не определено</t>
+          <t>медорганизация</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>аллергология, иммунология, анестезиология, реаниматология, гастроэнтерология, гинекология, дерматология, косметология, трихология, кардиология, неврология, онкология, оториноларингология, офтальмология, педиатрия, пульмонология, ревматология, терапия, урология, флебология, хирургия, эндокринология</t>
+          <t>флебология, хирургия</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
-          <t>Медицинский центр «Семья» в Ростове-на-Дону. Диагностика и лечение. Специальности врачей: аллерголог, гастроэнтеролог, гинеколог, дерматолог, косметолог, невролог, онколог, педиатр.</t>
+          <t>Лечение варикоза в Тольятти - приём флеболога, консультация 490 руб.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>АГАТ, ООО</t>
+          <t>АВТО-МЕД, ООО</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>6162081830</t>
+          <t>6324110942</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
@@ -21070,32 +21585,32 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>не определено</t>
+          <t>медорганизация</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>аллергология-иммунология, анестезиология-реаниматология</t>
+          <t>флебология</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>На сайте mc-semya.ru указаны страницы с услугами аллергологии-иммунологии и анестезиологии-реаниматологии, что является явным медицинским признаком.</t>
+          <t>Лечение варикоза в Тольятти - приём флеболога, консультация 490 руб.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>АГАТ, ООО</t>
+          <t>АВТО-МЕД, ООО</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>6162081830</t>
+          <t>6324110942</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
@@ -21110,32 +21625,32 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>не определено</t>
+          <t>медорганизация</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>аллергология-иммунология, анестезиология и реаниматология, гастроэнтерология, гинекология, дерматология, иммунология, кардиология, косметология, неврология, онкология, оториноларингология, офтальмология, педиатрия, пульмонология, ревматология, терапия, трихология, урология, флебология, хирургия, эндокринология</t>
+          <t>флебология, хирургия</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
-          <t>Медицинский центр «Семья» в Ростове-на-Дону. Диагностика и лечение.</t>
+          <t>Лечение варикоза в Тольятти - приём флеболога, консультация 490 руб!</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>АГК, ООО</t>
+          <t>АВТОРСКАЯ КЛИНИКА, ООО</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>2461016768</t>
+          <t>5407494063</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
@@ -21155,27 +21670,27 @@
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>Акушерство и гинекология, Андрология и урология, Лабораторная диагностика, Физиотерапия, Ультразвуковая диагностика, Хирургия, Сосудистая хирургия, Оперативная гинекология, Проктология, Эндоскопия, Маммология и онкология, Плазмолифтинг, Терапевт</t>
+          <t>пластическая хирургия, косметология, диетология, сомнология, мезотерапия, пилинг, инъекционная косметология, аппаратная косметология, хирургия груди, хирургия тела, хирургия лица, биоимпедансометрия, похудение</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>«Клиника лицензирована и соответствует всем требованиям медицинской безопасности»</t>
+          <t>Клиника пластической хирургии и врачебной косметологии в Новосибирске</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>АГК, ООО</t>
+          <t>АВТОРСКАЯ КЛИНИКА, ООО</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>2461016768</t>
+          <t>5407494063</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
@@ -21195,27 +21710,27 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>гинекология, урология, хирургия, онкология, терапия</t>
+          <t>косметология, пластическая хирургия</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>Услуги центра: Акушерство и гинекология, Андрология и Урология, Хирургия, Маммология и онкология, Терапевт</t>
+          <t>Лицензия №1, Приложение к лицензии №1, Приложение к лицензии №2-1, Приложение к лицензии №2-2, Приложение к лицензии №2-3, Лицензия №2</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>АГК, ООО</t>
+          <t>АВТОРСКАЯ КЛИНИКА, ООО</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>2461016768</t>
+          <t>5407494063</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
@@ -21235,27 +21750,27 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>акушерство и гинекология, андрология и урология, лабораторная диагностика, физиотерапия, ультразвуковая диагностика, хирургия, сосудистая хирургия, оперативная гинекология, проктология, эндоскопия, маммология и онкология, терапия</t>
+          <t>пластическая хирургия, врачебная косметология, диетология, сомнология</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>ООО 'АГК' - первая частная клиника в Красноярске, занимающаяся вопросами мужского и женского здоровья с 1997г. Клиника лицензирована и соответствует всем требованиям медицинской безопасности.</t>
+          <t>Клиника пластической хирургии и врачебной косметологии в Новосибирске</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>АЗБУКА ЗДОРОВЬЯ, ООО</t>
+          <t>АГАТ, ООО</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>7813610598</t>
+          <t>6162081830</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
@@ -21275,27 +21790,27 @@
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>Гастроэнтерология, Дерматология, Неврология, Отоларингология, Офтальмология, Педиатрия, Стоматология, Терапия, Хирургия, Эндокринология, УЗИ, ЭКГ, Мануальная терапия, Психиатрия детская</t>
+          <t>аллергология, иммунология, анестезиология, реаниматология, гастроэнтерология, гинекология, дерматология, косметология, трихология, кардиология, неврология, онкология, оториноларингология, офтальмология, педиатрия, пульмонология, ревматология, терапия, урология, флебология, хирургия, эндокринология</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
-          <t>Семейный медицинский центр предлагает медицинские услуги. Запись к врачу в регистратуре детской поликлиники района в Самаре.</t>
+          <t>Медицинский центр «Семья» в Ростове-на-Дону. Диагностика и лечение. Специальности врачей: аллерголог, гастроэнтеролог, гинеколог, дерматолог, косметолог, невролог, онколог, педиатр.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>АЗБУКА ЗДОРОВЬЯ, ООО</t>
+          <t>АГАТ, ООО</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>7813610598</t>
+          <t>6162081830</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
@@ -21315,27 +21830,27 @@
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>общая практика, дерматология, стоматология</t>
+          <t>аллергология-иммунология, анестезиология-реаниматология</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>Семейный медицинский центр Самара 🏥 | Детский развивающий клуб, Семейный медицинский центр предлагает медицинские услуги. Запись к врачу в регистратуре детской поликлиники района в Самаре.</t>
+          <t>На сайте mc-semya.ru указаны страницы с услугами аллергологии-иммунологии и анестезиологии-реаниматологии, что является явным медицинским признаком.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>АЗБУКА ЗДОРОВЬЯ, ООО</t>
+          <t>АГАТ, ООО</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>7813610598</t>
+          <t>6162081830</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
@@ -21355,27 +21870,27 @@
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>гастроэнтерология, дерматология, неврология, отоларингология, офтальмология, педиатрия, стоматология, терапия, хирургия, эндокринология</t>
+          <t>аллергология-иммунология, анестезиология и реаниматология, гастроэнтерология, гинекология, дерматология, иммунология, кардиология, косметология, неврология, онкология, оториноларингология, офтальмология, педиатрия, пульмонология, ревматология, терапия, трихология, урология, флебология, хирургия, эндокринология</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
-          <t>Детская поликлиника 🏥. Семейный медицинский центр предлагает медицинские услуги.</t>
+          <t>Медицинский центр «Семья» в Ростове-на-Дону. Диагностика и лечение.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>АЗБУКА ЗДОРОВЬЯ, ООО</t>
+          <t>АГК, ООО</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>6314040975</t>
+          <t>2461016768</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
@@ -21395,27 +21910,27 @@
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>Гастроэнтерология, Дерматология, Неврология, Отоларингология, Офтальмология, Педиатрия, Стоматология, Терапия, Хирургия, Эндокринология, Мануальная терапия, Психиатрия детская, УЗИ, ЭКГ</t>
+          <t>Акушерство и гинекология, Андрология и урология, Лабораторная диагностика, Физиотерапия, Ультразвуковая диагностика, Хирургия, Сосудистая хирургия, Оперативная гинекология, Проктология, Эндоскопия, Маммология и онкология, Плазмолифтинг, Терапевт</t>
         </is>
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>Семейный медицинский центр предлагает медицинские услуги. Запись к врачу в регистратуре детской поликлиники района в Самаре.</t>
+          <t>«Клиника лицензирована и соответствует всем требованиям медицинской безопасности»</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>АЗБУКА ЗДОРОВЬЯ, ООО</t>
+          <t>АГК, ООО</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>6314040975</t>
+          <t>2461016768</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
@@ -21435,50 +21950,410 @@
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>общая практика, дерматология, стоматология</t>
+          <t>гинекология, урология, хирургия, онкология, терапия</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t>Семейный медицинский центр Самара 🏥 | Детский развивающий клуб, Семейный медицинский центр предлагает медицинские услуги. Запись к врачу в регистратуре детской поликлиники района в Самаре.</t>
+          <t>Услуги центра: Акушерство и гинекология, Андрология и Урология, Хирургия, Маммология и онкология, Терапевт</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>АГК, ООО</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>2461016768</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>yandexgpt</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>акушерство и гинекология, андрология и урология, лабораторная диагностика, физиотерапия, ультразвуковая диагностика, хирургия, сосудистая хирургия, оперативная гинекология, проктология, эндоскопия, маммология и онкология, терапия</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>ООО 'АГК' - первая частная клиника в Красноярске, занимающаяся вопросами мужского и женского здоровья с 1997г. Клиника лицензирована и соответствует всем требованиям медицинской безопасности.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>АДРЕМ, ООО</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>5404465184</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>groq</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>управляющая компания сети клиник</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>аллерголог, гастроэнтеролог, гинеколог, дерматолог, иммунолог, кардиолог, косметолог, невролог, онколог, отоларинголог, оториноларинголог, офтальмолог, педиатр, психотерапевт, пульмонолог, ревматолог, стоматолог, терапевт, трихолог, уролог, хирург, эндокринолог</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="inlineStr">
+        <is>
+          <t>*   [Лицензия](https://smitra.ru/patients/yuridicheskaya-informatsiya/litsenziya-ooo-smk-smitra/ \"Лицензия\")</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>АДРЕМ, ООО</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>5404465184</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>llm7</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>управляющая компания сети клиник</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>дерматология, косметология, трихология</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>На сайте указаны специальности врачей, в том числе дерматолог, косметолог и трихолог, что является явным медицинским признаком.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>АДРЕМ, ООО</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>5404465184</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>yandexgpt</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>управляющая компания сети клиник</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>аллергология, гастроэнтерология, гинекология, дерматология, иммунология, кардиология, косметология, неврология, онкология, отоларингология, офтальмология, педиатрия, психотерапия, пульмонология, ревматология, стоматология, терапия, трихология, урология, хирургия, эндокринология</t>
+        </is>
+      </c>
+      <c r="H93" s="2" t="inlineStr">
+        <is>
+          <t>Лицензия (https://smitra.ru)</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>АЗБУКА ЗДОРОВЬЯ, ООО</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>7813610598</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>groq</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>Гастроэнтерология, Дерматология, Неврология, Отоларингология, Офтальмология, Педиатрия, Стоматология, Терапия, Хирургия, Эндокринология, УЗИ, ЭКГ, Мануальная терапия, Психиатрия детская</t>
+        </is>
+      </c>
+      <c r="H94" s="2" t="inlineStr">
+        <is>
+          <t>Семейный медицинский центр предлагает медицинские услуги. Запись к врачу в регистратуре детской поликлиники района в Самаре.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>АЗБУКА ЗДОРОВЬЯ, ООО</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>7813610598</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>llm7</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>общая практика, дерматология, стоматология</t>
+        </is>
+      </c>
+      <c r="H95" s="2" t="inlineStr">
+        <is>
+          <t>Семейный медицинский центр Самара 🏥 | Детский развивающий клуб, Семейный медицинский центр предлагает медицинские услуги. Запись к врачу в регистратуре детской поликлиники района в Самаре.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>АЗБУКА ЗДОРОВЬЯ, ООО</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>7813610598</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>yandexgpt</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>гастроэнтерология, дерматология, неврология, отоларингология, офтальмология, педиатрия, стоматология, терапия, хирургия, эндокринология</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
+          <t>Детская поликлиника 🏥. Семейный медицинский центр предлагает медицинские услуги.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
         <v>42</v>
       </c>
-      <c r="B90" s="2" t="inlineStr">
+      <c r="B97" s="2" t="inlineStr">
         <is>
           <t>АЗБУКА ЗДОРОВЬЯ, ООО</t>
         </is>
       </c>
-      <c r="C90" s="2" t="inlineStr">
+      <c r="C97" s="2" t="inlineStr">
         <is>
           <t>6314040975</t>
         </is>
       </c>
-      <c r="D90" s="2" t="inlineStr">
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>groq</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>Гастроэнтерология, Дерматология, Неврология, Отоларингология, Офтальмология, Педиатрия, Стоматология, Терапия, Хирургия, Эндокринология, Мануальная терапия, Психиатрия детская, УЗИ, ЭКГ</t>
+        </is>
+      </c>
+      <c r="H97" s="2" t="inlineStr">
+        <is>
+          <t>Семейный медицинский центр предлагает медицинские услуги. Запись к врачу в регистратуре детской поликлиники района в Самаре.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>АЗБУКА ЗДОРОВЬЯ, ООО</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>6314040975</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>llm7</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>медорганизация</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="G98" s="2" t="inlineStr">
+        <is>
+          <t>общая практика, дерматология, стоматология</t>
+        </is>
+      </c>
+      <c r="H98" s="2" t="inlineStr">
+        <is>
+          <t>Семейный медицинский центр Самара 🏥 | Детский развивающий клуб, Семейный медицинский центр предлагает медицинские услуги. Запись к врачу в регистратуре детской поликлиники района в Самаре.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>АЗБУКА ЗДОРОВЬЯ, ООО</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>6314040975</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
         <is>
           <t>yandexgpt</t>
         </is>
       </c>
-      <c r="E90" s="2" t="inlineStr">
+      <c r="E99" s="2" t="inlineStr">
         <is>
           <t>медорганизация</t>
         </is>
       </c>
-      <c r="F90" s="2" t="inlineStr">
+      <c r="F99" s="2" t="inlineStr">
         <is>
           <t>не определено</t>
         </is>
       </c>
-      <c r="G90" s="2" t="inlineStr">
+      <c r="G99" s="2" t="inlineStr">
         <is>
           <t>гастроэнтерология, дерматология, неврология, отоларингология, офтальмология, педиатрия, стоматология, терапия, хирургия, эндокринология</t>
         </is>
       </c>
-      <c r="H90" s="2" t="inlineStr">
+      <c r="H99" s="2" t="inlineStr">
         <is>
           <t>Детская поликлиника 🏥. Семейный медицинский центр предлагает медицинские услуги.</t>
         </is>
@@ -22373,13 +23248,29 @@
           <t>Челябинск</t>
         </is>
       </c>
-      <c r="O8" s="2" t="inlineStr"/>
-      <c r="P8" s="2" t="inlineStr"/>
-      <c r="Q8" s="2" t="inlineStr"/>
-      <c r="R8" s="2" t="inlineStr"/>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>a_medika.legal.invitro.ru</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>поиск (название+город, гибкая навигация)</t>
+        </is>
+      </c>
+      <c r="Q8" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён ИНН</t>
+        </is>
+      </c>
+      <c r="R8" s="2" t="inlineStr">
+        <is>
+          <t>ИНН 7453279603 найден на сайте</t>
+        </is>
+      </c>
       <c r="S8" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
+          <t>Сайт недоступен (уровни 1-4)</t>
         </is>
       </c>
       <c r="T8" s="2" t="inlineStr"/>
@@ -22390,7 +23281,9 @@
       <c r="Y8" s="2" t="inlineStr"/>
       <c r="Z8" s="2" t="inlineStr"/>
       <c r="AA8" s="2" t="inlineStr"/>
-      <c r="AB8" s="2" t="inlineStr"/>
+      <c r="AB8" s="2" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -22566,7 +23459,9 @@
       <c r="Y10" s="2" t="inlineStr"/>
       <c r="Z10" s="2" t="inlineStr"/>
       <c r="AA10" s="2" t="inlineStr"/>
-      <c r="AB10" s="2" t="inlineStr"/>
+      <c r="AB10" s="2" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -22931,24 +23826,70 @@
           <t>Самара</t>
         </is>
       </c>
-      <c r="O14" s="2" t="inlineStr"/>
-      <c r="P14" s="2" t="inlineStr"/>
-      <c r="Q14" s="2" t="inlineStr"/>
-      <c r="R14" s="2" t="inlineStr"/>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>samara.a2med.ru</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>поиск (название+город, гибкая навигация)</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён адресом лицензии</t>
+        </is>
+      </c>
+      <c r="R14" s="2" t="inlineStr">
+        <is>
+          <t>адрес места деятельности из лицензии РЗН («мичурина, 15») найден на сайте</t>
+        </is>
+      </c>
       <c r="S14" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
-        </is>
-      </c>
-      <c r="T14" s="2" t="inlineStr"/>
-      <c r="U14" s="2" t="inlineStr"/>
-      <c r="V14" s="2" t="inlineStr"/>
-      <c r="W14" s="2" t="inlineStr"/>
-      <c r="X14" s="2" t="inlineStr"/>
-      <c r="Y14" s="2" t="inlineStr"/>
-      <c r="Z14" s="2" t="inlineStr"/>
-      <c r="AA14" s="2" t="inlineStr"/>
-      <c r="AB14" s="2" t="inlineStr"/>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="T14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="U14" s="2" t="inlineStr">
+        <is>
+          <t>управляющая компания сети клиник</t>
+        </is>
+      </c>
+      <c r="V14" s="2" t="inlineStr">
+        <is>
+          <t>«…d.ru/about/news/deputat-samarskoj-gubernskoj-dumyi-nagradil-sotrudnikov-a2med-za-vklad-v-zdravooxranenie)  [![Image 32: Сеть медицинских центров A2MED успешно провела дебютный выпуск ЦФА](https://samara.a2med.ru/assets/components/phpthumbof/cache/f857ce1a6be64ef2e3a12a7e3650154e.e689433ec902b8707142247a8cb11e8c.jpg) 19.09.2024 #### Сеть медицинских центров A2MED успешно провела деб…» (https://samara.a2med.ru)</t>
+        </is>
+      </c>
+      <c r="W14" s="2" t="inlineStr">
+        <is>
+          <t>d.ru/about/news/deputat-samarskoj-gubernskoj-dumyi-nagradil-sotrudnikov-a2med-za-vklad-v-zdravooxranenie)  [![Image 32: Сеть медицинских центров A2MED успешно провела дебютный выпуск ЦФА](https://samara.a2med.ru/assets/components/phpthumbof/cache/f857ce1a6be64ef2e3a12a7e3650154e.e689433ec902b8707142</t>
+        </is>
+      </c>
+      <c r="X14" s="2" t="inlineStr">
+        <is>
+          <t>не похож</t>
+        </is>
+      </c>
+      <c r="Y14" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z14" s="2" t="inlineStr">
+        <is>
+          <t>[Код 06-036] Билирубин общий (Биохимия / Общий билирубин / Пигмент желчи, продукт распада гемоглобина); [Код 09-006] Epstein Barr Virus, ДНК [реал-тайм ПЦР] (Вирус инфекционного мононуклеоза / Вирус Эпштейна-Барр / ВЭБ / Герпес 4 типа, ДНК / Герпес-вирус 4 типа / Эпштейна-Барр)</t>
+        </is>
+      </c>
+      <c r="AA14" s="2" t="inlineStr">
+        <is>
+          <t>аллерголог, гастроэнтеролог, гинеколог, дерматолог, иммунолог, кардиолог, косметолог, невролог, онколог, оториноларинголог, офтальмолог, педиатр, ревматолог, стоматолог, терапевт, уролог, флеболог, хирург, эндокринолог</t>
+        </is>
+      </c>
+      <c r="AB14" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -23858,7 +24799,9 @@
       <c r="Y23" s="2" t="inlineStr"/>
       <c r="Z23" s="2" t="inlineStr"/>
       <c r="AA23" s="2" t="inlineStr"/>
-      <c r="AB23" s="2" t="inlineStr"/>
+      <c r="AB23" s="2" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -24539,24 +25482,58 @@
           <t>Ростов-на-Дону</t>
         </is>
       </c>
-      <c r="O30" s="2" t="inlineStr"/>
-      <c r="P30" s="2" t="inlineStr"/>
-      <c r="Q30" s="2" t="inlineStr"/>
-      <c r="R30" s="2" t="inlineStr"/>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>rpkavrora.clients.site</t>
+        </is>
+      </c>
+      <c r="P30" s="2" t="inlineStr">
+        <is>
+          <t>поиск (название+город, гибкая навигация)</t>
+        </is>
+      </c>
+      <c r="Q30" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён адресом</t>
+        </is>
+      </c>
+      <c r="R30" s="2" t="inlineStr">
+        <is>
+          <t>адрес организации в городе Ростов-на-Дону (контакт-блок/подвал); содержание соответствует названию</t>
+        </is>
+      </c>
       <c r="S30" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
-        </is>
-      </c>
-      <c r="T30" s="2" t="inlineStr"/>
-      <c r="U30" s="2" t="inlineStr"/>
-      <c r="V30" s="2" t="inlineStr"/>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="T30" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="U30" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="V30" s="2" t="inlineStr">
+        <is>
+          <t>медицинские слова есть, сильных оснований (лицензия с мед-контекстом / приём врача) нет</t>
+        </is>
+      </c>
       <c r="W30" s="2" t="inlineStr"/>
-      <c r="X30" s="2" t="inlineStr"/>
-      <c r="Y30" s="2" t="inlineStr"/>
+      <c r="X30" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="Y30" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="Z30" s="2" t="inlineStr"/>
       <c r="AA30" s="2" t="inlineStr"/>
-      <c r="AB30" s="2" t="inlineStr"/>
+      <c r="AB30" s="2" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -24994,7 +25971,9 @@
       <c r="Y35" s="2" t="inlineStr"/>
       <c r="Z35" s="2" t="inlineStr"/>
       <c r="AA35" s="2" t="inlineStr"/>
-      <c r="AB35" s="2" t="inlineStr"/>
+      <c r="AB35" s="2" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -25160,7 +26139,9 @@
       <c r="Y37" s="2" t="inlineStr"/>
       <c r="Z37" s="2" t="inlineStr"/>
       <c r="AA37" s="2" t="inlineStr"/>
-      <c r="AB37" s="2" t="inlineStr"/>
+      <c r="AB37" s="2" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -25331,24 +26312,66 @@
           <t>Новосибирск</t>
         </is>
       </c>
-      <c r="O39" s="2" t="inlineStr"/>
-      <c r="P39" s="2" t="inlineStr"/>
-      <c r="Q39" s="2" t="inlineStr"/>
-      <c r="R39" s="2" t="inlineStr"/>
+      <c r="O39" s="2" t="inlineStr">
+        <is>
+          <t>smitra.ru</t>
+        </is>
+      </c>
+      <c r="P39" s="2" t="inlineStr">
+        <is>
+          <t>поиск (название+город, гибкая навигация)</t>
+        </is>
+      </c>
+      <c r="Q39" s="2" t="inlineStr">
+        <is>
+          <t>подтверждён адресом лицензии</t>
+        </is>
+      </c>
+      <c r="R39" s="2" t="inlineStr">
+        <is>
+          <t>адрес места деятельности из лицензии РЗН («геодезическая, 2/1») найден на сайте</t>
+        </is>
+      </c>
       <c r="S39" s="2" t="inlineStr">
         <is>
-          <t>сайт не найден</t>
-        </is>
-      </c>
-      <c r="T39" s="2" t="inlineStr"/>
-      <c r="U39" s="2" t="inlineStr"/>
-      <c r="V39" s="2" t="inlineStr"/>
-      <c r="W39" s="2" t="inlineStr"/>
-      <c r="X39" s="2" t="inlineStr"/>
-      <c r="Y39" s="2" t="inlineStr"/>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="T39" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="U39" s="2" t="inlineStr">
+        <is>
+          <t>управляющая компания сети клиник</t>
+        </is>
+      </c>
+      <c r="V39" s="2" t="inlineStr">
+        <is>
+          <t>«…/news/cherno-belaya-vecherinka-kommersant-sibir-shakhmaty-klassika-i-zabota-o-zdorove-ot-kliniki-smitra/)  [![Image 55: Сеть клиник «Смитра» признана лучшей в здравоохранении на городском конкурсе](https://smitra.ru/upload/webp/upload/iblock/f1d/79x9y5vtvwfiecyksen2q2yv5k2aiqpa.webp)](https://smitra.ru/news/set-klinik-smitra-priznana-luchshey-v-zdravookhranenii-na-goro…» (https://smitra.ru)</t>
+        </is>
+      </c>
+      <c r="W39" s="2" t="inlineStr">
+        <is>
+          <t>/news/cherno-belaya-vecherinka-kommersant-sibir-shakhmaty-klassika-i-zabota-o-zdorove-ot-kliniki-smitra/)  [![Image 55: Сеть клиник «Смитра» признана лучшей в здравоохранении на городском конкурсе](https://smitra.ru/upload/webp/upload/iblock/f1d/79x9y5vtvwfiecyksen2q2yv5k2aiqpa.webp)](https://smitra</t>
+        </is>
+      </c>
+      <c r="X39" s="2" t="inlineStr">
+        <is>
+          <t>не определено</t>
+        </is>
+      </c>
+      <c r="Y39" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="Z39" s="2" t="inlineStr"/>
-      <c r="AA39" s="2" t="inlineStr"/>
-      <c r="AB39" s="2" t="inlineStr"/>
+      <c r="AA39" s="2" t="inlineStr">
+        <is>
+          <t>аллерголог, гастроэнтеролог, гинеколог, дерматолог, иммунолог, кардиолог, косметолог, невролог, онколог, отоларинголог, оториноларинголог, офтальмолог, педиатр, психотерапевт, пульмонолог, ревматолог, стоматолог, терапевт, трихолог, уролог, хирург, эндокринолог</t>
+        </is>
+      </c>
+      <c r="AB39" s="2" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">

</xml_diff>